<commit_message>
Meripurpuratus finalizado, arquivos echinatus baixados
</commit_message>
<xml_diff>
--- a/Ocorrências Literatura.xlsx
+++ b/Ocorrências Literatura.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faculdade\Laboratorio\lagostas_carapaca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1DE25C-A56E-41E4-9CB4-4A917A550F19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EEE8A1-169B-44F9-A319-6912070AF953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="143">
   <si>
     <t>origem</t>
   </si>
@@ -326,6 +326,147 @@
   </si>
   <si>
     <t>Cruz, R. (2025)</t>
+  </si>
+  <si>
+    <t>8°30′07″</t>
+  </si>
+  <si>
+    <t>35°00′08″</t>
+  </si>
+  <si>
+    <t>Porto de Galinhas</t>
+  </si>
+  <si>
+    <t>08°44′23″</t>
+  </si>
+  <si>
+    <t>35°02′28″</t>
+  </si>
+  <si>
+    <t>Tamandaré, PE</t>
+  </si>
+  <si>
+    <t>1-s2.0-S1470160X21011304-main</t>
+  </si>
+  <si>
+    <t>Giraldes, B (2021)</t>
+  </si>
+  <si>
+    <t>Guarapari (ES)</t>
+  </si>
+  <si>
+    <t>20°39′</t>
+  </si>
+  <si>
+    <t>40°30′</t>
+  </si>
+  <si>
+    <t>20°43′</t>
+  </si>
+  <si>
+    <t>40°46′</t>
+  </si>
+  <si>
+    <t>21°02′</t>
+  </si>
+  <si>
+    <t>40°49′</t>
+  </si>
+  <si>
+    <t>Anchieta (ES)</t>
+  </si>
+  <si>
+    <t>Marataízes (ES)</t>
+  </si>
+  <si>
+    <t>MELO, Andressa C. M. (2025)</t>
+  </si>
+  <si>
+    <t>Fisheries Management Eco - 2025 - Melo - Reproductive Biology of the Smoothtail Spiny Lobster  Panulirus laevicauda  to</t>
+  </si>
+  <si>
+    <t>São Pedro e São Paulo</t>
+  </si>
+  <si>
+    <t>0°55′10″</t>
+  </si>
+  <si>
+    <t>29°20′33″</t>
+  </si>
+  <si>
+    <t>0°54.787′</t>
+  </si>
+  <si>
+    <t>29°21.451′</t>
+  </si>
+  <si>
+    <t>0°55.681′</t>
+  </si>
+  <si>
+    <t>29°19.804′</t>
+  </si>
+  <si>
+    <t>Nunesetal2017DeepSeaDecapodCrustaceansSPSPA</t>
+  </si>
+  <si>
+    <t>NUNES, Diogo Martins (2017)</t>
+  </si>
+  <si>
+    <t>8°59′57″</t>
+  </si>
+  <si>
+    <t>35°10′49″</t>
+  </si>
+  <si>
+    <t>Alagoas (Maragogi / São José da Coroa Grande)</t>
+  </si>
+  <si>
+    <t>Bragrança</t>
+  </si>
+  <si>
+    <t>1°03′57″</t>
+  </si>
+  <si>
+    <t>46°47′22″W</t>
+  </si>
+  <si>
+    <t>PANAMJAS_16(2)_123-128</t>
+  </si>
+  <si>
+    <t>peerj-19586</t>
+  </si>
+  <si>
+    <t>GAETA, Juliana de Carvalho (2021)</t>
+  </si>
+  <si>
+    <t>SOUSA, Jefferson (2025)</t>
+  </si>
+  <si>
+    <t>Recife (PE)</t>
+  </si>
+  <si>
+    <t>08°10′</t>
+  </si>
+  <si>
+    <t>34°49′</t>
+  </si>
+  <si>
+    <t>s00435-019-00461-5</t>
+  </si>
+  <si>
+    <t>HAMILTON, Santiago (2019)</t>
+  </si>
+  <si>
+    <t>8°30′54″</t>
+  </si>
+  <si>
+    <t>34°59′47″</t>
+  </si>
+  <si>
+    <t>Giraldes, B (2012)</t>
+  </si>
+  <si>
+    <t>Composition and spatial distribution of subtidal Decapoda on the “Reef Coast”, northeastern Brazil, evaluated through a low-impact visual census technique</t>
   </si>
 </sst>
 </file>
@@ -482,7 +623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -553,6 +694,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -843,7 +987,7 @@
     <col min="4" max="4" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.28515625" style="3" customWidth="1"/>
     <col min="9" max="9" width="45" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="9.140625" style="3"/>
@@ -1383,7 +1527,7 @@
       <c r="H9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="20" t="s">
+      <c r="I9" s="25" t="s">
         <v>37</v>
       </c>
       <c r="J9" s="3" t="str">
@@ -2517,7 +2661,7 @@
       <c r="F27" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="8" t="s">
         <v>84</v>
       </c>
       <c r="H27" s="3" t="s">
@@ -2581,7 +2725,7 @@
       <c r="F28" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" s="8" t="s">
         <v>84</v>
       </c>
       <c r="H28" s="3" t="s">
@@ -2645,7 +2789,7 @@
       <c r="F29" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" s="8" t="s">
         <v>84</v>
       </c>
       <c r="H29" s="3" t="s">
@@ -2709,7 +2853,7 @@
       <c r="F30" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="8" t="s">
         <v>84</v>
       </c>
       <c r="H30" s="3" t="s">
@@ -2767,10 +2911,10 @@
       <c r="D31" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="8" t="s">
         <v>88</v>
       </c>
       <c r="G31" s="8" t="s">
@@ -2831,10 +2975,10 @@
       <c r="D32" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="8" t="s">
         <v>92</v>
       </c>
       <c r="G32" s="8" t="s">
@@ -2895,10 +3039,10 @@
       <c r="D33" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="8" t="s">
         <v>94</v>
       </c>
       <c r="G33" s="8" t="s">
@@ -2907,7 +3051,9 @@
       <c r="H33" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I33" s="5"/>
+      <c r="I33" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="J33" s="3" t="str">
         <f t="shared" si="24"/>
         <v>3</v>
@@ -2944,210 +3090,309 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
+      <c r="B34" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C34" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I34" s="5"/>
-      <c r="J34" s="3" t="e">
+      <c r="E34" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J34" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K34" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K34" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L34" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L34" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M34" s="3" t="e">
+        <v>07</v>
+      </c>
+      <c r="M34" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N34" s="3" t="e">
+        <v>35</v>
+      </c>
+      <c r="N34" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O34" s="3" t="e">
+        <v>00</v>
+      </c>
+      <c r="O34" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P34" s="1" t="e">
+        <v>08</v>
+      </c>
+      <c r="P34" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q34" s="1" t="e">
+        <v>-8.5019444444444439</v>
+      </c>
+      <c r="Q34" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-35.002222222222223</v>
+      </c>
+      <c r="R34" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
+      <c r="B35" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C35" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I35" s="5"/>
-      <c r="J35" s="3" t="e">
+      <c r="E35" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J35" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K35" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K35" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L35" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L35" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M35" s="3" t="e">
+        <v>07</v>
+      </c>
+      <c r="M35" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N35" s="3" t="e">
+        <v>35</v>
+      </c>
+      <c r="N35" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O35" s="3" t="e">
+        <v>00</v>
+      </c>
+      <c r="O35" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P35" s="1" t="e">
+        <v>08</v>
+      </c>
+      <c r="P35" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q35" s="1" t="e">
+        <v>-8.5019444444444439</v>
+      </c>
+      <c r="Q35" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-35.002222222222223</v>
+      </c>
+      <c r="R35" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
+      <c r="B36" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="C36" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I36" s="5"/>
-      <c r="J36" s="3" t="e">
+      <c r="E36" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J36" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K36" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K36" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L36" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L36" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M36" s="3" t="e">
+        <v>07</v>
+      </c>
+      <c r="M36" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N36" s="3" t="e">
+        <v>35</v>
+      </c>
+      <c r="N36" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O36" s="3" t="e">
+        <v>00</v>
+      </c>
+      <c r="O36" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P36" s="1" t="e">
+        <v>08</v>
+      </c>
+      <c r="P36" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q36" s="1" t="e">
+        <v>-8.5019444444444439</v>
+      </c>
+      <c r="Q36" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-35.002222222222223</v>
+      </c>
+      <c r="R36" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
+      <c r="B37" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C37" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J37" s="3" t="e">
+      <c r="E37" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J37" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K37" s="3" t="e">
+        <v>08</v>
+      </c>
+      <c r="K37" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L37" s="3" t="e">
+        <v>44</v>
+      </c>
+      <c r="L37" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M37" s="3" t="e">
+        <v>23</v>
+      </c>
+      <c r="M37" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N37" s="3" t="e">
+        <v>35</v>
+      </c>
+      <c r="N37" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O37" s="3" t="e">
+        <v>02</v>
+      </c>
+      <c r="O37" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P37" s="1" t="e">
+        <v>28</v>
+      </c>
+      <c r="P37" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q37" s="1" t="e">
+        <v>-8.7397222222222215</v>
+      </c>
+      <c r="Q37" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-35.041111111111114</v>
+      </c>
+      <c r="R37" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
+      <c r="B38" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C38" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J38" s="3" t="e">
+      <c r="E38" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="J38" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K38" s="3" t="e">
+        <v>20</v>
+      </c>
+      <c r="K38" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>39</v>
       </c>
       <c r="L38" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M38" s="3" t="e">
+      <c r="M38" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N38" s="3" t="e">
+        <v>40</v>
+      </c>
+      <c r="N38" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>30</v>
       </c>
       <c r="O38" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3161,36 +3406,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R38" s="14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
+      <c r="B39" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C39" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J39" s="3" t="e">
+      <c r="E39" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G39" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I39" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="J39" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K39" s="3" t="e">
+        <v>20</v>
+      </c>
+      <c r="K39" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>43</v>
       </c>
       <c r="L39" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M39" s="3" t="e">
+      <c r="M39" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N39" s="3" t="e">
+        <v>40</v>
+      </c>
+      <c r="N39" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>46</v>
       </c>
       <c r="O39" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3204,36 +3470,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R39" s="14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
+      <c r="B40" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C40" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J40" s="3" t="e">
+      <c r="E40" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="J40" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K40" s="3" t="e">
+        <v>21</v>
+      </c>
+      <c r="K40" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>02</v>
       </c>
       <c r="L40" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M40" s="3" t="e">
+      <c r="M40" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N40" s="3" t="e">
+        <v>40</v>
+      </c>
+      <c r="N40" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>49</v>
       </c>
       <c r="O40" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3247,81 +3534,121 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R40" s="14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
+      <c r="B41" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C41" s="3" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I41" s="5"/>
-      <c r="J41" s="3" t="e">
+      <c r="E41" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J41" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K41" s="3" t="e">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L41" s="3" t="e">
+        <v>55</v>
+      </c>
+      <c r="L41" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M41" s="3" t="e">
+        <v>10</v>
+      </c>
+      <c r="M41" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N41" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="N41" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O41" s="3" t="e">
+        <v>20</v>
+      </c>
+      <c r="O41" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P41" s="1" t="e">
+        <v>33</v>
+      </c>
+      <c r="P41" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q41" s="1" t="e">
+        <v>0.9194444444444444</v>
+      </c>
+      <c r="Q41" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-29.342500000000001</v>
+      </c>
+      <c r="R41" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
+      <c r="B42" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C42" s="3" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I42" s="5"/>
-      <c r="J42" s="3" t="e">
+      <c r="E42" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J42" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K42" s="3" t="e">
+        <v>0</v>
+      </c>
+      <c r="K42" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>54.787</v>
       </c>
       <c r="L42" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M42" s="3" t="e">
+      <c r="M42" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N42" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="N42" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>21.451</v>
       </c>
       <c r="O42" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3335,37 +3662,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R42" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
+      <c r="B43" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C43" s="3" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I43" s="5"/>
-      <c r="J43" s="3" t="e">
+      <c r="E43" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J43" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K43" s="3" t="e">
+        <v>0</v>
+      </c>
+      <c r="K43" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>55.681</v>
       </c>
       <c r="L43" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M43" s="3" t="e">
+      <c r="M43" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N43" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="N43" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>19.804</v>
       </c>
       <c r="O43" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3379,80 +3726,121 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R43" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
+      <c r="B44" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C44" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I44" s="5"/>
-      <c r="J44" s="3" t="e">
+      <c r="E44" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J44" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K44" s="3" t="e">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L44" s="3" t="e">
+        <v>55</v>
+      </c>
+      <c r="L44" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M44" s="3" t="e">
+        <v>10</v>
+      </c>
+      <c r="M44" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N44" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="N44" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O44" s="3" t="e">
+        <v>20</v>
+      </c>
+      <c r="O44" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P44" s="1" t="e">
+        <v>33</v>
+      </c>
+      <c r="P44" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q44" s="1" t="e">
+        <v>-0.9194444444444444</v>
+      </c>
+      <c r="Q44" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-29.342500000000001</v>
+      </c>
+      <c r="R44" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
+      <c r="B45" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C45" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J45" s="3" t="e">
+      <c r="E45" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G45" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J45" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K45" s="3" t="e">
+        <v>0</v>
+      </c>
+      <c r="K45" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>54.787</v>
       </c>
       <c r="L45" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M45" s="3" t="e">
+      <c r="M45" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N45" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="N45" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>21.451</v>
       </c>
       <c r="O45" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3466,36 +3854,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R45" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
+      <c r="B46" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C46" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J46" s="3" t="e">
+      <c r="E46" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G46" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J46" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K46" s="3" t="e">
+        <v>0</v>
+      </c>
+      <c r="K46" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>55.681</v>
       </c>
       <c r="L46" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M46" s="3" t="e">
+      <c r="M46" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N46" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="N46" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>19.804</v>
       </c>
       <c r="O46" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3509,167 +3918,249 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R46" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
+      <c r="B47" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C47" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J47" s="3" t="e">
+      <c r="E47" t="s">
+        <v>124</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G47" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="J47" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K47" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K47" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L47" s="3" t="e">
+        <v>59</v>
+      </c>
+      <c r="L47" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M47" s="3" t="e">
+        <v>57</v>
+      </c>
+      <c r="M47" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N47" s="3" t="e">
+        <v>35</v>
+      </c>
+      <c r="N47" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O47" s="3" t="e">
+        <v>10</v>
+      </c>
+      <c r="O47" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P47" s="1" t="e">
+        <v>49</v>
+      </c>
+      <c r="P47" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q47" s="1" t="e">
+        <v>-8.9991666666666674</v>
+      </c>
+      <c r="Q47" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-35.180277777777775</v>
+      </c>
+      <c r="R47" s="14" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
+      <c r="B48" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="C48" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J48" s="3" t="e">
+      <c r="E48" t="s">
+        <v>128</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J48" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K48" s="3" t="e">
+        <v>1</v>
+      </c>
+      <c r="K48" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L48" s="3" t="e">
+        <v>03</v>
+      </c>
+      <c r="L48" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M48" s="3" t="e">
+        <v>57</v>
+      </c>
+      <c r="M48" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N48" s="3" t="e">
+        <v>46</v>
+      </c>
+      <c r="N48" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O48" s="3" t="e">
+        <v>47</v>
+      </c>
+      <c r="O48" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P48" s="1" t="e">
+        <v>22</v>
+      </c>
+      <c r="P48" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q48" s="1" t="e">
+        <v>-1.0658333333333334</v>
+      </c>
+      <c r="Q48" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-46.789444444444442</v>
+      </c>
+      <c r="R48" s="14" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
+      <c r="B49" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C49" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I49" s="5"/>
-      <c r="J49" s="3" t="e">
+      <c r="E49" t="s">
+        <v>128</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J49" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K49" s="3" t="e">
+        <v>1</v>
+      </c>
+      <c r="K49" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L49" s="3" t="e">
+        <v>03</v>
+      </c>
+      <c r="L49" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M49" s="3" t="e">
+        <v>57</v>
+      </c>
+      <c r="M49" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N49" s="3" t="e">
+        <v>46</v>
+      </c>
+      <c r="N49" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O49" s="3" t="e">
+        <v>47</v>
+      </c>
+      <c r="O49" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P49" s="1" t="e">
+        <v>22</v>
+      </c>
+      <c r="P49" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q49" s="1" t="e">
+        <v>-1.0658333333333334</v>
+      </c>
+      <c r="Q49" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-46.789444444444442</v>
+      </c>
+      <c r="R49" s="14" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
+      <c r="B50" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C50" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I50" s="5"/>
-      <c r="J50" s="3" t="e">
+      <c r="E50" t="s">
+        <v>135</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G50" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J50" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K50" s="3" t="e">
+        <v>08</v>
+      </c>
+      <c r="K50" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>10</v>
       </c>
       <c r="L50" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M50" s="3" t="e">
+      <c r="M50" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N50" s="3" t="e">
+        <v>34</v>
+      </c>
+      <c r="N50" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>49</v>
       </c>
       <c r="O50" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3683,37 +4174,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R50" s="14" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>50</v>
       </c>
+      <c r="B51" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="C51" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I51" s="5"/>
-      <c r="J51" s="3" t="e">
+      <c r="E51" t="s">
+        <v>135</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J51" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K51" s="3" t="e">
+        <v>08</v>
+      </c>
+      <c r="K51" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>10</v>
       </c>
       <c r="L51" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M51" s="3" t="e">
+      <c r="M51" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N51" s="3" t="e">
+        <v>34</v>
+      </c>
+      <c r="N51" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>49</v>
       </c>
       <c r="O51" s="3" t="e">
         <f t="shared" si="29"/>
@@ -3727,141 +4238,203 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R51" s="14" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>51</v>
       </c>
+      <c r="B52" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C52" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I52" s="5"/>
-      <c r="J52" s="3" t="e">
+      <c r="E52" t="s">
+        <v>139</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J52" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K52" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K52" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L52" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L52" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M52" s="3" t="e">
+        <v>54</v>
+      </c>
+      <c r="M52" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N52" s="3" t="e">
+        <v>34</v>
+      </c>
+      <c r="N52" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O52" s="3" t="e">
+        <v>59</v>
+      </c>
+      <c r="O52" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P52" s="1" t="e">
+        <v>47</v>
+      </c>
+      <c r="P52" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q52" s="1" t="e">
+        <v>-8.5150000000000006</v>
+      </c>
+      <c r="Q52" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-34.996388888888887</v>
+      </c>
+      <c r="R52" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>52</v>
       </c>
+      <c r="B53" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C53" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="J53" s="3" t="e">
+      <c r="E53" t="s">
+        <v>139</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J53" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K53" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K53" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L53" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L53" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M53" s="3" t="e">
+        <v>54</v>
+      </c>
+      <c r="M53" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N53" s="3" t="e">
+        <v>34</v>
+      </c>
+      <c r="N53" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O53" s="3" t="e">
+        <v>59</v>
+      </c>
+      <c r="O53" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P53" s="1" t="e">
+        <v>47</v>
+      </c>
+      <c r="P53" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q53" s="1" t="e">
+        <v>-8.5150000000000006</v>
+      </c>
+      <c r="Q53" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-34.996388888888887</v>
+      </c>
+      <c r="R53" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>53</v>
       </c>
+      <c r="B54" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C54" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E54" s="2"/>
-      <c r="J54" s="3" t="e">
+      <c r="E54" t="s">
+        <v>139</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J54" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K54" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K54" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L54" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L54" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M54" s="3" t="e">
+        <v>54</v>
+      </c>
+      <c r="M54" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N54" s="3" t="e">
+        <v>34</v>
+      </c>
+      <c r="N54" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O54" s="3" t="e">
+        <v>59</v>
+      </c>
+      <c r="O54" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P54" s="1" t="e">
+        <v>47</v>
+      </c>
+      <c r="P54" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q54" s="1" t="e">
+        <v>-8.5150000000000006</v>
+      </c>
+      <c r="Q54" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-34.996388888888887</v>
+      </c>
+      <c r="R54" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -3905,8 +4478,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R55" s="14"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -3951,7 +4525,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -3996,7 +4570,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -4041,7 +4615,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -4086,7 +4660,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -4131,7 +4705,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -4176,7 +4750,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -4221,7 +4795,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>62</v>
       </c>
@@ -4266,7 +4840,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
Finalizando o Fim de semana
</commit_message>
<xml_diff>
--- a/Ocorrências Literatura.xlsx
+++ b/Ocorrências Literatura.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faculdade\Laboratorio\lagostas_carapaca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EEE8A1-169B-44F9-A319-6912070AF953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04A7F3C-0B61-4FF5-AA07-AB2615B93860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="178">
   <si>
     <t>origem</t>
   </si>
@@ -467,13 +467,153 @@
   </si>
   <si>
     <t>Composition and spatial distribution of subtidal Decapoda on the “Reef Coast”, northeastern Brazil, evaluated through a low-impact visual census technique</t>
+  </si>
+  <si>
+    <t>18°01′15″</t>
+  </si>
+  <si>
+    <t>38°43′16″</t>
+  </si>
+  <si>
+    <t>Arquipélogo de Abrolhos (BA)</t>
+  </si>
+  <si>
+    <t>Belém (PA)</t>
+  </si>
+  <si>
+    <t>São Paulo Capital (SP)</t>
+  </si>
+  <si>
+    <t>01°27′</t>
+  </si>
+  <si>
+    <t>48°30′</t>
+  </si>
+  <si>
+    <t>23°32′</t>
+  </si>
+  <si>
+    <t>46°38′</t>
+  </si>
+  <si>
+    <t>03°50′</t>
+  </si>
+  <si>
+    <t>38°20′</t>
+  </si>
+  <si>
+    <t>23°17′</t>
+  </si>
+  <si>
+    <t>44°10′</t>
+  </si>
+  <si>
+    <r>
+      <t>Baía da Ilha Grande</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, no litoral sul do Rio de Janeiro (Costa Verde).</t>
+    </r>
+  </si>
+  <si>
+    <t>Região costeira do Ceará, nas proximidades de Aquiraz</t>
+  </si>
+  <si>
+    <t>4°25′</t>
+  </si>
+  <si>
+    <t>37°16′</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Litoral leste do </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ceará</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, na região de Aracati (próximo ao estuário do Rio Jaguaribe).</t>
+    </r>
+  </si>
+  <si>
+    <t>Santa Barbara Island</t>
+  </si>
+  <si>
+    <t>Redonda Island</t>
+  </si>
+  <si>
+    <t>Siriba Island</t>
+  </si>
+  <si>
+    <t>FARIA JÚNIOR, Edson (2013)</t>
+  </si>
+  <si>
+    <t>1.pdf</t>
+  </si>
+  <si>
+    <t>17°57′29″</t>
+  </si>
+  <si>
+    <t>38°42′09″</t>
+  </si>
+  <si>
+    <t>17°57′38″</t>
+  </si>
+  <si>
+    <t>38°42′55″</t>
+  </si>
+  <si>
+    <t>17°57′59″</t>
+  </si>
+  <si>
+    <t>38°42′52″</t>
+  </si>
+  <si>
+    <t>32°24′</t>
+  </si>
+  <si>
+    <t>Arquipélago de Fernando de Noronha</t>
+  </si>
+  <si>
+    <t>03°45′</t>
+  </si>
+  <si>
+    <t>32°19′</t>
+  </si>
+  <si>
+    <t>Atol das Rocas</t>
+  </si>
+  <si>
+    <t>1-s2.0-S2351989415001031-main</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,6 +693,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -623,7 +778,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -697,6 +852,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3935,7 +4093,7 @@
       <c r="D47" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="8" t="s">
         <v>124</v>
       </c>
       <c r="F47" s="1" t="s">
@@ -3999,7 +4157,7 @@
       <c r="D48" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" s="8" t="s">
         <v>128</v>
       </c>
       <c r="F48" s="1" t="s">
@@ -4063,7 +4221,7 @@
       <c r="D49" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="8" t="s">
         <v>128</v>
       </c>
       <c r="F49" s="1" t="s">
@@ -4127,7 +4285,7 @@
       <c r="D50" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" s="8" t="s">
         <v>135</v>
       </c>
       <c r="F50" s="1" t="s">
@@ -4191,7 +4349,7 @@
       <c r="D51" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="8" t="s">
         <v>135</v>
       </c>
       <c r="F51" s="1" t="s">
@@ -4255,7 +4413,7 @@
       <c r="D52" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E52" s="8" t="s">
         <v>139</v>
       </c>
       <c r="F52" s="1" t="s">
@@ -4319,7 +4477,7 @@
       <c r="D53" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" s="8" t="s">
         <v>139</v>
       </c>
       <c r="F53" s="1" t="s">
@@ -4383,7 +4541,7 @@
       <c r="D54" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E54" s="8" t="s">
         <v>139</v>
       </c>
       <c r="F54" s="1" t="s">
@@ -4438,169 +4596,241 @@
       <c r="A55" s="3">
         <v>54</v>
       </c>
+      <c r="B55" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C55" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="J55" s="3" t="e">
+      <c r="E55" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="F55" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="J55" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K55" s="3" t="e">
+        <v>18</v>
+      </c>
+      <c r="K55" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L55" s="3" t="e">
+        <v>01</v>
+      </c>
+      <c r="L55" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M55" s="3" t="e">
+        <v>15</v>
+      </c>
+      <c r="M55" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N55" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N55" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O55" s="3" t="e">
+        <v>43</v>
+      </c>
+      <c r="O55" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P55" s="1" t="e">
+        <v>16</v>
+      </c>
+      <c r="P55" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q55" s="1" t="e">
+        <v>-18.020833333333332</v>
+      </c>
+      <c r="Q55" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="R55" s="14"/>
-    </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-38.721111111111114</v>
+      </c>
+      <c r="R55" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
+      <c r="B56" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C56" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="J56" s="3" t="e">
+      <c r="E56" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="J56" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K56" s="3" t="e">
+        <v>18</v>
+      </c>
+      <c r="K56" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L56" s="3" t="e">
+        <v>01</v>
+      </c>
+      <c r="L56" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M56" s="3" t="e">
+        <v>15</v>
+      </c>
+      <c r="M56" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N56" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N56" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O56" s="3" t="e">
+        <v>43</v>
+      </c>
+      <c r="O56" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P56" s="1" t="e">
+        <v>16</v>
+      </c>
+      <c r="P56" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q56" s="1" t="e">
+        <v>-18.020833333333332</v>
+      </c>
+      <c r="Q56" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-38.721111111111114</v>
+      </c>
+      <c r="R56" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
+      <c r="B57" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C57" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="J57" s="3" t="e">
+      <c r="E57" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="F57" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="J57" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K57" s="3" t="e">
+        <v>18</v>
+      </c>
+      <c r="K57" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L57" s="3" t="e">
+        <v>01</v>
+      </c>
+      <c r="L57" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M57" s="3" t="e">
+        <v>15</v>
+      </c>
+      <c r="M57" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N57" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N57" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O57" s="3" t="e">
+        <v>43</v>
+      </c>
+      <c r="O57" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P57" s="1" t="e">
+        <v>16</v>
+      </c>
+      <c r="P57" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q57" s="1" t="e">
+        <v>-18.020833333333332</v>
+      </c>
+      <c r="Q57" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-38.721111111111114</v>
+      </c>
+      <c r="R57" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
+      <c r="B58" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C58" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
-      <c r="J58" s="3" t="e">
+      <c r="E58" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="J58" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K58" s="3" t="e">
+        <v>01</v>
+      </c>
+      <c r="K58" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>27</v>
       </c>
       <c r="L58" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M58" s="3" t="e">
+      <c r="M58" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N58" s="3" t="e">
+        <v>48</v>
+      </c>
+      <c r="N58" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>30</v>
       </c>
       <c r="O58" s="3" t="e">
         <f t="shared" si="29"/>
@@ -4614,38 +4844,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R58" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
+      <c r="B59" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C59" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
-      <c r="J59" s="3" t="e">
+      <c r="E59" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="G59" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="J59" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K59" s="3" t="e">
+        <v>23</v>
+      </c>
+      <c r="K59" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>32</v>
       </c>
       <c r="L59" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M59" s="3" t="e">
+      <c r="M59" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N59" s="3" t="e">
+        <v>46</v>
+      </c>
+      <c r="N59" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>38</v>
       </c>
       <c r="O59" s="3" t="e">
         <f t="shared" si="29"/>
@@ -4659,38 +4908,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R59" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
+      <c r="B60" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C60" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="J60" s="3" t="e">
+      <c r="E60" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I60" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="J60" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K60" s="3" t="e">
+        <v>03</v>
+      </c>
+      <c r="K60" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>50</v>
       </c>
       <c r="L60" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M60" s="3" t="e">
+      <c r="M60" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N60" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N60" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>20</v>
       </c>
       <c r="O60" s="3" t="e">
         <f t="shared" si="29"/>
@@ -4704,38 +4972,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R60" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
+      <c r="B61" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C61" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="J61" s="3" t="e">
+      <c r="E61" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="G61" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I61" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="J61" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K61" s="3" t="e">
+        <v>23</v>
+      </c>
+      <c r="K61" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>17</v>
       </c>
       <c r="L61" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M61" s="3" t="e">
+      <c r="M61" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N61" s="3" t="e">
+        <v>44</v>
+      </c>
+      <c r="N61" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>10</v>
       </c>
       <c r="O61" s="3" t="e">
         <f t="shared" si="29"/>
@@ -4749,38 +5036,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R61" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
+      <c r="B62" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C62" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="J62" s="3" t="e">
+      <c r="E62" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I62" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="J62" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K62" s="3" t="e">
+        <v>4</v>
+      </c>
+      <c r="K62" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>25</v>
       </c>
       <c r="L62" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M62" s="3" t="e">
+      <c r="M62" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N62" s="3" t="e">
+        <v>37</v>
+      </c>
+      <c r="N62" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>16</v>
       </c>
       <c r="O62" s="3" t="e">
         <f t="shared" si="29"/>
@@ -4794,173 +5100,249 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R62" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>62</v>
       </c>
+      <c r="B63" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C63" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-      <c r="J63" s="3" t="e">
+      <c r="E63" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F63" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="G63" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="J63" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K63" s="3" t="e">
+        <v>17</v>
+      </c>
+      <c r="K63" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L63" s="3" t="e">
+        <v>57</v>
+      </c>
+      <c r="L63" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M63" s="3" t="e">
+        <v>29</v>
+      </c>
+      <c r="M63" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N63" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N63" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O63" s="3" t="e">
+        <v>42</v>
+      </c>
+      <c r="O63" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P63" s="1" t="e">
+        <v>09</v>
+      </c>
+      <c r="P63" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q63" s="1" t="e">
+        <v>-17.958055555555557</v>
+      </c>
+      <c r="Q63" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+        <v>-38.702500000000001</v>
+      </c>
+      <c r="R63" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>63</v>
       </c>
+      <c r="B64" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C64" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="J64" s="3" t="e">
+      <c r="E64" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="F64" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="J64" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K64" s="3" t="e">
+        <v>17</v>
+      </c>
+      <c r="K64" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L64" s="3" t="e">
+        <v>57</v>
+      </c>
+      <c r="L64" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M64" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="M64" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N64" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N64" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O64" s="3" t="e">
+        <v>42</v>
+      </c>
+      <c r="O64" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P64" s="1" t="e">
+        <v>55</v>
+      </c>
+      <c r="P64" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q64" s="1" t="e">
+        <v>-17.960555555555555</v>
+      </c>
+      <c r="Q64" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-38.715277777777779</v>
+      </c>
+      <c r="R64" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>64</v>
       </c>
+      <c r="B65" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="C65" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="J65" s="3" t="e">
+      <c r="E65" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F65" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="G65" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="J65" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K65" s="3" t="e">
+        <v>17</v>
+      </c>
+      <c r="K65" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L65" s="3" t="e">
+        <v>57</v>
+      </c>
+      <c r="L65" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M65" s="3" t="e">
+        <v>59</v>
+      </c>
+      <c r="M65" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N65" s="3" t="e">
+        <v>38</v>
+      </c>
+      <c r="N65" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O65" s="3" t="e">
+        <v>42</v>
+      </c>
+      <c r="O65" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P65" s="1" t="e">
+        <v>52</v>
+      </c>
+      <c r="P65" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q65" s="1" t="e">
+        <v>-17.96638888888889</v>
+      </c>
+      <c r="Q65" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-38.714444444444446</v>
+      </c>
+      <c r="R65" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>65</v>
       </c>
+      <c r="B66" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C66" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
-      <c r="J66" s="3" t="e">
+      <c r="E66" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I66" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="J66" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K66" s="3" t="e">
+        <v>03</v>
+      </c>
+      <c r="K66" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>50</v>
       </c>
       <c r="L66" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M66" s="3" t="e">
+      <c r="M66" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N66" s="3" t="e">
+        <v>32</v>
+      </c>
+      <c r="N66" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>24</v>
       </c>
       <c r="O66" s="3" t="e">
         <f t="shared" si="29"/>
@@ -4974,38 +5356,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R66" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>66</v>
       </c>
+      <c r="B67" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="C67" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-      <c r="J67" s="3" t="e">
+      <c r="E67" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I67" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="J67" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K67" s="3" t="e">
+        <v>03</v>
+      </c>
+      <c r="K67" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>45</v>
       </c>
       <c r="L67" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M67" s="3" t="e">
+      <c r="M67" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N67" s="3" t="e">
+        <v>32</v>
+      </c>
+      <c r="N67" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>19</v>
       </c>
       <c r="O67" s="3" t="e">
         <f t="shared" si="29"/>
@@ -5019,37 +5420,57 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R67" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="68" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
+      <c r="B68" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C68" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E68" s="2"/>
-      <c r="J68" s="3" t="e">
+      <c r="E68" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I68" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="J68" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K68" s="3" t="e">
+        <v>03</v>
+      </c>
+      <c r="K68" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
+        <v>50</v>
       </c>
       <c r="L68" s="3" t="e">
         <f t="shared" si="26"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M68" s="3" t="e">
+      <c r="M68" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N68" s="3" t="e">
+        <v>32</v>
+      </c>
+      <c r="N68" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
+        <v>24</v>
       </c>
       <c r="O68" s="3" t="e">
         <f t="shared" si="29"/>
@@ -5063,8 +5484,11 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R68" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -5074,42 +5498,55 @@
       <c r="D69" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="J69" s="3" t="e">
+      <c r="E69" t="s">
+        <v>139</v>
+      </c>
+      <c r="F69" t="s">
+        <v>140</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J69" s="3" t="str">
         <f t="shared" si="24"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K69" s="3" t="e">
+        <v>8</v>
+      </c>
+      <c r="K69" s="3" t="str">
         <f t="shared" si="25"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L69" s="3" t="e">
+        <v>30</v>
+      </c>
+      <c r="L69" s="3" t="str">
         <f t="shared" si="26"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M69" s="3" t="e">
+        <v>54</v>
+      </c>
+      <c r="M69" s="3" t="str">
         <f t="shared" si="27"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N69" s="3" t="e">
+        <v>34</v>
+      </c>
+      <c r="N69" s="3" t="str">
         <f t="shared" si="28"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O69" s="3" t="e">
+        <v>59</v>
+      </c>
+      <c r="O69" s="3" t="str">
         <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P69" s="1" t="e">
+        <v>47</v>
+      </c>
+      <c r="P69" s="1">
         <f t="shared" si="30"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q69" s="1" t="e">
+        <v>-8.5150000000000006</v>
+      </c>
+      <c r="Q69" s="1">
         <f t="shared" si="31"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+        <v>-34.996388888888887</v>
+      </c>
+      <c r="R69" s="14" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -5153,8 +5590,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R70" s="14"/>
+    </row>
+    <row r="71" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>70</v>
       </c>
@@ -5198,8 +5636,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R71" s="14"/>
+    </row>
+    <row r="72" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>71</v>
       </c>
@@ -5243,8 +5682,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R72" s="14"/>
+    </row>
+    <row r="73" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>72</v>
       </c>
@@ -5287,8 +5727,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R73" s="14"/>
+    </row>
+    <row r="74" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>73</v>
       </c>
@@ -5330,8 +5771,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R74" s="14"/>
+    </row>
+    <row r="75" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>74</v>
       </c>
@@ -5373,8 +5815,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R75" s="14"/>
+    </row>
+    <row r="76" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>75</v>
       </c>
@@ -5416,8 +5859,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R76" s="14"/>
+    </row>
+    <row r="77" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>76</v>
       </c>
@@ -5459,8 +5903,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R77" s="14"/>
+    </row>
+    <row r="78" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>77</v>
       </c>
@@ -5502,8 +5947,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R78" s="14"/>
+    </row>
+    <row r="79" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>78</v>
       </c>
@@ -5545,8 +5991,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R79" s="14"/>
+    </row>
+    <row r="80" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>79</v>
       </c>
@@ -5588,8 +6035,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R80" s="14"/>
+    </row>
+    <row r="81" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -5631,8 +6079,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R81" s="14"/>
+    </row>
+    <row r="82" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -5674,8 +6123,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R82" s="14"/>
+    </row>
+    <row r="83" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -5717,8 +6167,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R83" s="14"/>
+    </row>
+    <row r="84" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -5760,8 +6211,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R84" s="14"/>
+    </row>
+    <row r="85" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>84</v>
       </c>
@@ -5803,8 +6255,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R85" s="14"/>
+    </row>
+    <row r="86" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>85</v>
       </c>
@@ -5846,8 +6299,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R86" s="14"/>
+    </row>
+    <row r="87" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>86</v>
       </c>
@@ -5889,8 +6343,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R87" s="14"/>
+    </row>
+    <row r="88" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>87</v>
       </c>
@@ -5932,8 +6387,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R88" s="14"/>
+    </row>
+    <row r="89" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>88</v>
       </c>
@@ -5975,8 +6431,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R89" s="14"/>
+    </row>
+    <row r="90" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>89</v>
       </c>
@@ -6018,8 +6475,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R90" s="14"/>
+    </row>
+    <row r="91" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>90</v>
       </c>
@@ -6061,8 +6519,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R91" s="14"/>
+    </row>
+    <row r="92" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>91</v>
       </c>
@@ -6104,8 +6563,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R92" s="14"/>
+    </row>
+    <row r="93" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>92</v>
       </c>
@@ -6147,8 +6607,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R93" s="14"/>
+    </row>
+    <row r="94" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>93</v>
       </c>
@@ -6190,8 +6651,9 @@
         <f t="shared" si="31"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R94" s="14"/>
+    </row>
+    <row r="95" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>94</v>
       </c>
@@ -6233,8 +6695,9 @@
         <f t="shared" ref="Q95:Q140" si="39">((((O95/60)+N95)/60)+M95)*IF(D95="W",-1, 1)</f>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R95" s="14"/>
+    </row>
+    <row r="96" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>95</v>
       </c>
@@ -6276,8 +6739,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R96" s="14"/>
+    </row>
+    <row r="97" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>96</v>
       </c>
@@ -6319,8 +6783,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R97" s="14"/>
+    </row>
+    <row r="98" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>97</v>
       </c>
@@ -6362,8 +6827,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R98" s="14"/>
+    </row>
+    <row r="99" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>98</v>
       </c>
@@ -6405,8 +6871,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R99" s="14"/>
+    </row>
+    <row r="100" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>99</v>
       </c>
@@ -6448,8 +6915,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R100" s="14"/>
+    </row>
+    <row r="101" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>100</v>
       </c>
@@ -6491,8 +6959,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R101" s="14"/>
+    </row>
+    <row r="102" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>101</v>
       </c>
@@ -6534,8 +7003,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R102" s="14"/>
+    </row>
+    <row r="103" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>102</v>
       </c>
@@ -6577,8 +7047,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R103" s="14"/>
+    </row>
+    <row r="104" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>103</v>
       </c>
@@ -6620,8 +7091,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R104" s="14"/>
+    </row>
+    <row r="105" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>104</v>
       </c>
@@ -6664,8 +7136,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R105" s="14"/>
+    </row>
+    <row r="106" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>105</v>
       </c>
@@ -6708,8 +7181,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R106" s="14"/>
+    </row>
+    <row r="107" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>106</v>
       </c>
@@ -6752,8 +7226,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R107" s="14"/>
+    </row>
+    <row r="108" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>107</v>
       </c>
@@ -6795,8 +7270,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R108" s="14"/>
+    </row>
+    <row r="109" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>108</v>
       </c>
@@ -6838,8 +7314,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R109" s="14"/>
+    </row>
+    <row r="110" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>109</v>
       </c>
@@ -6881,8 +7358,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R110" s="14"/>
+    </row>
+    <row r="111" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>110</v>
       </c>
@@ -6924,8 +7402,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R111" s="14"/>
+    </row>
+    <row r="112" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>111</v>
       </c>
@@ -6967,8 +7446,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R112" s="14"/>
+    </row>
+    <row r="113" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>112</v>
       </c>
@@ -7010,8 +7490,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R113" s="14"/>
+    </row>
+    <row r="114" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>113</v>
       </c>
@@ -7054,8 +7535,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R114" s="14"/>
+    </row>
+    <row r="115" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>114</v>
       </c>
@@ -7098,8 +7580,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R115" s="14"/>
+    </row>
+    <row r="116" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>115</v>
       </c>
@@ -7142,8 +7625,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R116" s="14"/>
+    </row>
+    <row r="117" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>116</v>
       </c>
@@ -7186,8 +7670,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R117" s="14"/>
+    </row>
+    <row r="118" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>117</v>
       </c>
@@ -7229,8 +7714,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R118" s="14"/>
+    </row>
+    <row r="119" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>118</v>
       </c>
@@ -7272,8 +7758,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R119" s="14"/>
+    </row>
+    <row r="120" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>119</v>
       </c>
@@ -7315,8 +7802,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R120" s="14"/>
+    </row>
+    <row r="121" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>120</v>
       </c>
@@ -7358,8 +7846,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R121" s="14"/>
+    </row>
+    <row r="122" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>121</v>
       </c>
@@ -7401,8 +7890,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R122" s="14"/>
+    </row>
+    <row r="123" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>122</v>
       </c>
@@ -7444,8 +7934,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R123" s="14"/>
+    </row>
+    <row r="124" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
         <v>123</v>
       </c>
@@ -7487,8 +7978,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R124" s="14"/>
+    </row>
+    <row r="125" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
         <v>124</v>
       </c>
@@ -7530,8 +8022,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R125" s="14"/>
+    </row>
+    <row r="126" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
         <v>125</v>
       </c>
@@ -7573,8 +8066,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R126" s="14"/>
+    </row>
+    <row r="127" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
         <v>126</v>
       </c>
@@ -7616,8 +8110,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R127" s="14"/>
+    </row>
+    <row r="128" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
         <v>127</v>
       </c>
@@ -7659,8 +8154,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R128" s="14"/>
+    </row>
+    <row r="129" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
         <v>128</v>
       </c>
@@ -7703,8 +8199,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R129" s="14"/>
+    </row>
+    <row r="130" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
         <v>129</v>
       </c>
@@ -7747,8 +8244,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R130" s="14"/>
+    </row>
+    <row r="131" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
         <v>130</v>
       </c>
@@ -7790,8 +8288,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R131" s="14"/>
+    </row>
+    <row r="132" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="3">
         <v>131</v>
       </c>
@@ -7833,8 +8332,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R132" s="14"/>
+    </row>
+    <row r="133" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="3">
         <v>132</v>
       </c>
@@ -7876,8 +8376,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R133" s="14"/>
+    </row>
+    <row r="134" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="3">
         <v>133</v>
       </c>
@@ -7919,8 +8420,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R134" s="14"/>
+    </row>
+    <row r="135" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
         <v>134</v>
       </c>
@@ -7962,8 +8464,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R135" s="14"/>
+    </row>
+    <row r="136" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
         <v>135</v>
       </c>
@@ -8005,8 +8508,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R136" s="14"/>
+    </row>
+    <row r="137" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
         <v>136</v>
       </c>
@@ -8048,8 +8552,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R137" s="14"/>
+    </row>
+    <row r="138" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" s="3">
         <v>137</v>
       </c>
@@ -8093,8 +8598,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R138" s="14"/>
+    </row>
+    <row r="139" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
         <v>138</v>
       </c>
@@ -8138,8 +8644,9 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R139" s="14"/>
+    </row>
+    <row r="140" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" s="3">
         <v>139</v>
       </c>
@@ -8183,22 +8690,23 @@
         <f t="shared" si="39"/>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R140" s="14"/>
+    </row>
+    <row r="141" spans="1:18" x14ac:dyDescent="0.25">
       <c r="E141" s="2"/>
       <c r="F141" s="2"/>
       <c r="P141" s="1"/>
       <c r="Q141" s="1"/>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P142" s="1"/>
       <c r="Q142" s="1"/>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P143" s="1"/>
       <c r="Q143" s="1"/>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P144" s="1"/>
       <c r="Q144" s="1"/>
     </row>

</xml_diff>

<commit_message>
Finalizando o levantamento de dados de ocorrência
</commit_message>
<xml_diff>
--- a/Ocorrências Literatura.xlsx
+++ b/Ocorrências Literatura.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faculdade\Laboratorio\lagostas_carapaca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EA36930-029B-40E9-8259-A5AF32AA04D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F921765-7979-4B94-9560-399387C6944E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Ocorrências Panulirus" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$B$1:$I$477</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ocorrências Panulirus'!$B$1:$I$477</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1032,7 +1032,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1108,13 +1108,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>

</xml_diff>

<commit_message>
Dados Google Earth Pro
</commit_message>
<xml_diff>
--- a/Ocorrências Literatura.xlsx
+++ b/Ocorrências Literatura.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faculdade\Laboratorio\lagostas_carapaca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DEC900-C0A2-4462-B6BE-81BAD4D6D2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074B4B81-D42B-4B22-B984-4BA5AC186470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2129,7 +2129,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R466"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2150,7 +2149,7 @@
     <col min="19" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -2206,7 +2205,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.6" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -2270,7 +2269,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="33">
         <v>2</v>
       </c>
@@ -2334,7 +2333,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33">
         <v>3</v>
       </c>
@@ -2398,7 +2397,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="33">
         <v>4</v>
       </c>
@@ -2462,7 +2461,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="33">
         <v>5</v>
       </c>
@@ -2526,7 +2525,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="33">
         <v>6</v>
       </c>
@@ -2590,7 +2589,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="33">
         <v>7</v>
       </c>
@@ -2654,7 +2653,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="33">
         <v>8</v>
       </c>
@@ -2718,7 +2717,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="33">
         <v>9</v>
       </c>
@@ -2782,7 +2781,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="33">
         <v>10</v>
       </c>
@@ -2846,7 +2845,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" s="33">
         <v>11</v>
       </c>
@@ -2910,7 +2909,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A13" s="33">
         <v>12</v>
       </c>
@@ -2974,7 +2973,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A14" s="33">
         <v>13</v>
       </c>
@@ -3038,7 +3037,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" s="33">
         <v>14</v>
       </c>
@@ -3102,7 +3101,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="33">
         <v>15</v>
       </c>
@@ -3294,7 +3293,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="33">
         <v>18</v>
       </c>
@@ -3358,7 +3357,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="33">
         <v>19</v>
       </c>
@@ -3422,7 +3421,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="33">
         <v>20</v>
       </c>
@@ -3486,7 +3485,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="33">
         <v>21</v>
       </c>
@@ -3550,7 +3549,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="33">
         <v>22</v>
       </c>
@@ -3614,7 +3613,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="33">
         <v>23</v>
       </c>
@@ -3678,7 +3677,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="33">
         <v>24</v>
       </c>
@@ -3742,7 +3741,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="33">
         <v>25</v>
       </c>
@@ -3806,7 +3805,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="33">
         <v>26</v>
       </c>
@@ -3870,7 +3869,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="33">
         <v>27</v>
       </c>
@@ -3998,7 +3997,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="33">
         <v>29</v>
       </c>
@@ -4062,7 +4061,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="33">
         <v>30</v>
       </c>
@@ -4126,7 +4125,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="33">
         <v>31</v>
       </c>
@@ -4190,7 +4189,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="33">
         <v>32</v>
       </c>
@@ -4254,7 +4253,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="33">
         <v>33</v>
       </c>
@@ -4318,7 +4317,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="33">
         <v>34</v>
       </c>
@@ -4382,7 +4381,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="33">
         <v>35</v>
       </c>
@@ -4446,7 +4445,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="33">
         <v>36</v>
       </c>
@@ -4510,7 +4509,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="33">
         <v>37</v>
       </c>
@@ -4574,7 +4573,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="33">
         <v>38</v>
       </c>
@@ -4638,7 +4637,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="33">
         <v>39</v>
       </c>
@@ -4766,7 +4765,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="33">
         <v>41</v>
       </c>
@@ -4830,7 +4829,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="33">
         <v>42</v>
       </c>
@@ -4958,7 +4957,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="33">
         <v>44</v>
       </c>
@@ -5022,7 +5021,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="33">
         <v>45</v>
       </c>
@@ -5086,7 +5085,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="33">
         <v>46</v>
       </c>
@@ -5150,7 +5149,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="33">
         <v>47</v>
       </c>
@@ -5214,7 +5213,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="33">
         <v>48</v>
       </c>
@@ -5278,7 +5277,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="33">
         <v>49</v>
       </c>
@@ -5342,7 +5341,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="33">
         <v>50</v>
       </c>
@@ -5406,7 +5405,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="33">
         <v>51</v>
       </c>
@@ -5470,7 +5469,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="33">
         <v>52</v>
       </c>
@@ -5534,7 +5533,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="33">
         <v>53</v>
       </c>
@@ -5598,7 +5597,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="33">
         <v>54</v>
       </c>
@@ -5662,7 +5661,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="33">
         <v>55</v>
       </c>
@@ -5726,7 +5725,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="33">
         <v>56</v>
       </c>
@@ -5790,7 +5789,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="33">
         <v>57</v>
       </c>
@@ -5854,7 +5853,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="33">
         <v>58</v>
       </c>
@@ -5918,7 +5917,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="33">
         <v>59</v>
       </c>
@@ -5982,7 +5981,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="33">
         <v>60</v>
       </c>
@@ -6046,7 +6045,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="33">
         <v>61</v>
       </c>
@@ -6110,7 +6109,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="33">
         <v>62</v>
       </c>
@@ -6174,7 +6173,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="33">
         <v>63</v>
       </c>
@@ -6238,7 +6237,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="33">
         <v>64</v>
       </c>
@@ -6302,7 +6301,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="33">
         <v>65</v>
       </c>
@@ -6366,7 +6365,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="33">
         <v>66</v>
       </c>
@@ -6430,7 +6429,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="33">
         <v>67</v>
       </c>
@@ -6494,7 +6493,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="33">
         <v>68</v>
       </c>
@@ -6558,7 +6557,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="33">
         <v>69</v>
       </c>
@@ -6622,7 +6621,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="33">
         <v>70</v>
       </c>
@@ -6686,7 +6685,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="33">
         <v>71</v>
       </c>
@@ -6750,7 +6749,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="33">
         <v>72</v>
       </c>
@@ -6814,7 +6813,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="33">
         <v>73</v>
       </c>
@@ -6878,7 +6877,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="33">
         <v>74</v>
       </c>
@@ -6942,7 +6941,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="33">
         <v>75</v>
       </c>
@@ -7006,7 +7005,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="33">
         <v>76</v>
       </c>
@@ -7070,7 +7069,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="33">
         <v>77</v>
       </c>
@@ -7134,7 +7133,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="33">
         <v>78</v>
       </c>
@@ -7198,7 +7197,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="33">
         <v>79</v>
       </c>
@@ -7262,7 +7261,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="33">
         <v>80</v>
       </c>
@@ -7326,7 +7325,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="33">
         <v>81</v>
       </c>
@@ -7390,7 +7389,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="33">
         <v>82</v>
       </c>
@@ -7454,7 +7453,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="33">
         <v>83</v>
       </c>
@@ -7518,7 +7517,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="33">
         <v>84</v>
       </c>
@@ -7582,7 +7581,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="33">
         <v>85</v>
       </c>
@@ -7646,7 +7645,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="33">
         <v>86</v>
       </c>
@@ -7710,7 +7709,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="33">
         <v>87</v>
       </c>
@@ -7774,7 +7773,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="33">
         <v>88</v>
       </c>
@@ -7838,7 +7837,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="33">
         <v>89</v>
       </c>
@@ -7902,7 +7901,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="33">
         <v>90</v>
       </c>
@@ -7966,7 +7965,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="33">
         <v>91</v>
       </c>
@@ -8030,7 +8029,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="33">
         <v>92</v>
       </c>
@@ -8094,7 +8093,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="33">
         <v>93</v>
       </c>
@@ -8158,7 +8157,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="33">
         <v>94</v>
       </c>
@@ -8222,7 +8221,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="33">
         <v>95</v>
       </c>
@@ -8286,7 +8285,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="97" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="33">
         <v>96</v>
       </c>
@@ -8350,7 +8349,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="33">
         <v>97</v>
       </c>
@@ -8414,7 +8413,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="33">
         <v>98</v>
       </c>
@@ -8478,7 +8477,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="33">
         <v>99</v>
       </c>
@@ -8542,7 +8541,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="33">
         <v>100</v>
       </c>
@@ -8606,7 +8605,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="33">
         <v>101</v>
       </c>
@@ -8670,7 +8669,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="103" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" s="33">
         <v>102</v>
       </c>
@@ -8734,7 +8733,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" s="33">
         <v>103</v>
       </c>
@@ -8798,7 +8797,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" s="33">
         <v>104</v>
       </c>
@@ -8862,7 +8861,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="33">
         <v>105</v>
       </c>
@@ -8926,7 +8925,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="33">
         <v>106</v>
       </c>
@@ -8990,7 +8989,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="108" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="33">
         <v>107</v>
       </c>
@@ -9054,7 +9053,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="109" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="33">
         <v>108</v>
       </c>
@@ -9118,7 +9117,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="33">
         <v>109</v>
       </c>
@@ -9182,7 +9181,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="33">
         <v>110</v>
       </c>
@@ -9246,7 +9245,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="33">
         <v>111</v>
       </c>
@@ -9310,7 +9309,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="33">
         <v>112</v>
       </c>
@@ -9374,7 +9373,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="33">
         <v>113</v>
       </c>
@@ -9438,7 +9437,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="33">
         <v>114</v>
       </c>
@@ -9502,7 +9501,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="33">
         <v>115</v>
       </c>
@@ -9566,7 +9565,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="33">
         <v>116</v>
       </c>
@@ -9630,7 +9629,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="33">
         <v>117</v>
       </c>
@@ -9694,7 +9693,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="33">
         <v>118</v>
       </c>
@@ -9758,7 +9757,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="33">
         <v>119</v>
       </c>
@@ -10142,7 +10141,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="33">
         <v>125</v>
       </c>
@@ -10206,7 +10205,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="33">
         <v>126</v>
       </c>
@@ -10270,7 +10269,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="128" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="33">
         <v>127</v>
       </c>
@@ -10334,7 +10333,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A129" s="33">
         <v>128</v>
       </c>
@@ -10398,7 +10397,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="130" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" s="33">
         <v>129</v>
       </c>
@@ -10462,7 +10461,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" s="33">
         <v>130</v>
       </c>
@@ -10526,7 +10525,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="33">
         <v>131</v>
       </c>
@@ -10590,7 +10589,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="33">
         <v>132</v>
       </c>
@@ -10654,7 +10653,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="33">
         <v>133</v>
       </c>
@@ -10718,7 +10717,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="33">
         <v>134</v>
       </c>
@@ -10782,7 +10781,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="33">
         <v>135</v>
       </c>
@@ -10846,7 +10845,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" s="33">
         <v>136</v>
       </c>
@@ -10910,7 +10909,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" s="33">
         <v>137</v>
       </c>
@@ -10974,7 +10973,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" s="33">
         <v>138</v>
       </c>
@@ -11038,7 +11037,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="140" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" s="33">
         <v>139</v>
       </c>
@@ -11102,7 +11101,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" s="33">
         <v>140</v>
       </c>
@@ -11166,7 +11165,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A142" s="33">
         <v>141</v>
       </c>
@@ -11230,7 +11229,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" s="33">
         <v>142</v>
       </c>
@@ -11294,7 +11293,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A144" s="33">
         <v>143</v>
       </c>
@@ -11358,7 +11357,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A145" s="33">
         <v>144</v>
       </c>
@@ -11422,7 +11421,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="146" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A146" s="33">
         <v>145</v>
       </c>
@@ -11486,7 +11485,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" s="33">
         <v>146</v>
       </c>
@@ -11550,7 +11549,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" s="33">
         <v>147</v>
       </c>
@@ -11614,7 +11613,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="149" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" s="33">
         <v>148</v>
       </c>
@@ -11678,7 +11677,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A150" s="33">
         <v>149</v>
       </c>
@@ -11742,7 +11741,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" s="33">
         <v>150</v>
       </c>
@@ -11806,7 +11805,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="152" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" s="33">
         <v>151</v>
       </c>
@@ -11870,7 +11869,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="153" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" s="33">
         <v>152</v>
       </c>
@@ -11934,7 +11933,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="154" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A154" s="33">
         <v>153</v>
       </c>
@@ -11998,7 +11997,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="155" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A155" s="33">
         <v>154</v>
       </c>
@@ -12062,7 +12061,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="156" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A156" s="33">
         <v>155</v>
       </c>
@@ -12126,7 +12125,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="157" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A157" s="33">
         <v>156</v>
       </c>
@@ -12190,7 +12189,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="158" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A158" s="33">
         <v>157</v>
       </c>
@@ -12254,7 +12253,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="159" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A159" s="33">
         <v>158</v>
       </c>
@@ -12318,7 +12317,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="160" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A160" s="33">
         <v>159</v>
       </c>
@@ -12382,7 +12381,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="161" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A161" s="33">
         <v>160</v>
       </c>
@@ -12446,7 +12445,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="162" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A162" s="33">
         <v>161</v>
       </c>
@@ -12510,7 +12509,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="163" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A163" s="33">
         <v>162</v>
       </c>
@@ -12574,7 +12573,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="164" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A164" s="33">
         <v>163</v>
       </c>
@@ -12638,7 +12637,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="165" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A165" s="33">
         <v>164</v>
       </c>
@@ -12702,7 +12701,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="166" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A166" s="33">
         <v>165</v>
       </c>
@@ -12766,7 +12765,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="167" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A167" s="33">
         <v>166</v>
       </c>
@@ -12830,7 +12829,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="168" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A168" s="33">
         <v>167</v>
       </c>
@@ -12894,7 +12893,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="169" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A169" s="33">
         <v>168</v>
       </c>
@@ -12958,7 +12957,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="170" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A170" s="33">
         <v>169</v>
       </c>
@@ -13022,7 +13021,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="171" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A171" s="33">
         <v>170</v>
       </c>
@@ -13086,7 +13085,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="172" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A172" s="33">
         <v>171</v>
       </c>
@@ -13150,7 +13149,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="173" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A173" s="33">
         <v>172</v>
       </c>
@@ -13214,7 +13213,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="174" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A174" s="33">
         <v>173</v>
       </c>
@@ -13278,7 +13277,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="175" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A175" s="33">
         <v>174</v>
       </c>
@@ -13342,7 +13341,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A176" s="33">
         <v>175</v>
       </c>
@@ -13406,7 +13405,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="177" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A177" s="33">
         <v>176</v>
       </c>
@@ -13470,7 +13469,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="178" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A178" s="33">
         <v>177</v>
       </c>
@@ -13534,7 +13533,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="179" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A179" s="33">
         <v>178</v>
       </c>
@@ -13598,7 +13597,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="180" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A180" s="33">
         <v>179</v>
       </c>
@@ -13662,7 +13661,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="181" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A181" s="33">
         <v>180</v>
       </c>
@@ -13726,7 +13725,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="182" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A182" s="33">
         <v>181</v>
       </c>
@@ -13790,7 +13789,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="183" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A183" s="33">
         <v>182</v>
       </c>
@@ -13854,7 +13853,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="184" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A184" s="33">
         <v>183</v>
       </c>
@@ -13918,7 +13917,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A185" s="33">
         <v>184</v>
       </c>
@@ -13982,7 +13981,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="186" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A186" s="33">
         <v>185</v>
       </c>
@@ -14046,7 +14045,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="187" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A187" s="33">
         <v>186</v>
       </c>
@@ -14110,7 +14109,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="188" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A188" s="33">
         <v>187</v>
       </c>
@@ -14174,7 +14173,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="189" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A189" s="33">
         <v>188</v>
       </c>
@@ -14238,7 +14237,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="190" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A190" s="33">
         <v>189</v>
       </c>
@@ -14302,7 +14301,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="191" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A191" s="33">
         <v>190</v>
       </c>
@@ -14366,7 +14365,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="192" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A192" s="33">
         <v>191</v>
       </c>
@@ -14430,7 +14429,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="193" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A193" s="33">
         <v>192</v>
       </c>
@@ -14494,7 +14493,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="194" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A194" s="33">
         <v>193</v>
       </c>
@@ -14558,7 +14557,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="195" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A195" s="33">
         <v>194</v>
       </c>
@@ -14622,7 +14621,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="196" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A196" s="33">
         <v>195</v>
       </c>
@@ -14686,7 +14685,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="197" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A197" s="33">
         <v>196</v>
       </c>
@@ -14750,7 +14749,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="198" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A198" s="33">
         <v>197</v>
       </c>
@@ -14814,7 +14813,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="199" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A199" s="33">
         <v>198</v>
       </c>
@@ -14878,7 +14877,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="200" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A200" s="33">
         <v>199</v>
       </c>
@@ -14942,7 +14941,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="201" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A201" s="33">
         <v>200</v>
       </c>
@@ -15006,7 +15005,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="202" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A202" s="33">
         <v>201</v>
       </c>
@@ -15070,7 +15069,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="203" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A203" s="33">
         <v>202</v>
       </c>
@@ -15134,7 +15133,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="204" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A204" s="33">
         <v>203</v>
       </c>
@@ -15198,7 +15197,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="205" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A205" s="33">
         <v>204</v>
       </c>
@@ -15262,7 +15261,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="206" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A206" s="33">
         <v>205</v>
       </c>
@@ -15326,7 +15325,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="207" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A207" s="33">
         <v>206</v>
       </c>
@@ -15390,7 +15389,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="208" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A208" s="33">
         <v>207</v>
       </c>
@@ -15454,7 +15453,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="209" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A209" s="33">
         <v>208</v>
       </c>
@@ -15518,7 +15517,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="210" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A210" s="33">
         <v>209</v>
       </c>
@@ -15582,7 +15581,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="211" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A211" s="33">
         <v>210</v>
       </c>
@@ -15646,7 +15645,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="212" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A212" s="33">
         <v>211</v>
       </c>
@@ -15710,7 +15709,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="213" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A213" s="33">
         <v>212</v>
       </c>
@@ -15774,7 +15773,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="214" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A214" s="33">
         <v>213</v>
       </c>
@@ -15838,7 +15837,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="215" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A215" s="33">
         <v>214</v>
       </c>
@@ -15902,7 +15901,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="216" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A216" s="33">
         <v>215</v>
       </c>
@@ -16094,7 +16093,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="219" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A219" s="33">
         <v>218</v>
       </c>
@@ -16158,7 +16157,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="220" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A220" s="33">
         <v>219</v>
       </c>
@@ -16222,7 +16221,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="221" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A221" s="33">
         <v>220</v>
       </c>
@@ -16286,7 +16285,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="222" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A222" s="33">
         <v>221</v>
       </c>
@@ -17825,13 +17824,7 @@
       <c r="Q466" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:I222" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Panulirus meripurpuratus"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:I222" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Revsão dos dados baixados par P. guttatus
</commit_message>
<xml_diff>
--- a/Ocorrências Literatura.xlsx
+++ b/Ocorrências Literatura.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faculdade\Laboratorio\lagostas_carapaca\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cofres Obsidian\Mar Aberto\Laboratório\lagostas_carapaca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52A23E7-CDBD-46DA-B734-EBC2597E977E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC19BE9-1E65-4CCB-9247-0BF9A3CE5693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Planilha1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ocorrências Panulirus'!$B$1:$I$314</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ocorrências Panulirus'!$A$1:$R$387</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3239" uniqueCount="698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3815" uniqueCount="699">
   <si>
     <t>ID</t>
   </si>
@@ -2296,6 +2296,9 @@
   </si>
   <si>
     <t>15°51′53″</t>
+  </si>
+  <si>
+    <t>Panulirus guttatus</t>
   </si>
 </sst>
 </file>
@@ -8811,7 +8814,7 @@
         <v>17</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>19</v>
@@ -8857,7 +8860,7 @@
       </c>
       <c r="P95" s="2">
         <f t="shared" si="14"/>
-        <v>-20.85</v>
+        <v>20.85</v>
       </c>
       <c r="Q95" s="2">
         <f t="shared" si="15"/>
@@ -22912,31 +22915,31 @@
         <v>670</v>
       </c>
       <c r="J315" s="1" t="str">
-        <f t="shared" ref="J315:J323" si="56">MID(E315,1,FIND("°",E315,1)-1)</f>
+        <f t="shared" ref="J315:J378" si="56">MID(E315,1,FIND("°",E315,1)-1)</f>
         <v>12</v>
       </c>
       <c r="K315" s="1" t="str">
-        <f t="shared" ref="K315:K323" si="57">MID(E315,FIND("°",E315,1)+1,(FIND("′",E315,1)-FIND("°",E315,1))-1)</f>
+        <f t="shared" ref="K315:K378" si="57">MID(E315,FIND("°",E315,1)+1,(FIND("′",E315,1)-FIND("°",E315,1))-1)</f>
         <v>24</v>
       </c>
       <c r="L315" s="1" t="str">
-        <f t="shared" ref="L315:L323" si="58">MID(E315,FIND("′",E315,1)+1,(FIND("″",E315,1)-FIND("′",E315,1))-1)</f>
+        <f t="shared" ref="L315:L378" si="58">MID(E315,FIND("′",E315,1)+1,(FIND("″",E315,1)-FIND("′",E315,1))-1)</f>
         <v>56</v>
       </c>
       <c r="M315" s="1" t="str">
-        <f t="shared" ref="M315:M323" si="59">MID(F315,1,FIND("°",F315,1)-1)</f>
+        <f t="shared" ref="M315:M378" si="59">MID(F315,1,FIND("°",F315,1)-1)</f>
         <v>81</v>
       </c>
       <c r="N315" s="1" t="str">
-        <f t="shared" ref="N315:N323" si="60">MID(F315,FIND("°",F315,1)+1,(FIND("′",F315,1)-FIND("°",F315,1))-1)</f>
+        <f t="shared" ref="N315:N378" si="60">MID(F315,FIND("°",F315,1)+1,(FIND("′",F315,1)-FIND("°",F315,1))-1)</f>
         <v>28</v>
       </c>
       <c r="O315" s="1" t="str">
-        <f t="shared" ref="O315:O323" si="61">MID(F315,FIND("′",F315,1)+1,(FIND("″",F315,1)-FIND("′",F315,1))-1)</f>
+        <f t="shared" ref="O315:O378" si="61">MID(F315,FIND("′",F315,1)+1,(FIND("″",F315,1)-FIND("′",F315,1))-1)</f>
         <v>28</v>
       </c>
       <c r="P315" s="2">
-        <f t="shared" ref="P315:P323" si="62">((((L315/60)+K315)/60)+J315)*IF(C315="S",-1, 1)</f>
+        <f t="shared" ref="P315:P378" si="62">((((L315/60)+K315)/60)+J315)*IF(C315="S",-1, 1)</f>
         <v>12.415555555555555</v>
       </c>
       <c r="Q315" s="2">
@@ -23453,315 +23456,4109 @@
       </c>
       <c r="Q323" s="2">
         <f t="shared" si="63"/>
-        <v>81.849999999999994</v>
+        <v>-81.849999999999994</v>
       </c>
       <c r="R323" s="16" t="s">
         <v>679</v>
       </c>
     </row>
     <row r="324" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="P324" s="2"/>
-      <c r="Q324" s="2"/>
-      <c r="R324" s="16"/>
-    </row>
-    <row r="325" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P325" s="2"/>
-      <c r="Q325" s="2"/>
-    </row>
-    <row r="326" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P326" s="2"/>
-      <c r="Q326" s="2"/>
-    </row>
-    <row r="327" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P327" s="2"/>
-      <c r="Q327" s="2"/>
-    </row>
-    <row r="328" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P328" s="2"/>
-      <c r="Q328" s="2"/>
-    </row>
-    <row r="329" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P329" s="2"/>
-      <c r="Q329" s="2"/>
-    </row>
-    <row r="330" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P330" s="2"/>
-      <c r="Q330" s="2"/>
-    </row>
-    <row r="331" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P331" s="2"/>
-      <c r="Q331" s="2"/>
-    </row>
-    <row r="332" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P332" s="2"/>
-      <c r="Q332" s="2"/>
-    </row>
-    <row r="333" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P333" s="2"/>
-      <c r="Q333" s="2"/>
-    </row>
-    <row r="334" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P334" s="2"/>
-      <c r="Q334" s="2"/>
-    </row>
-    <row r="335" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P335" s="2"/>
-      <c r="Q335" s="2"/>
+      <c r="A324" s="1">
+        <v>323</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C324" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D324" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E324" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="F324" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="G324" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H324" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I324" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="J324" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K324" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>31</v>
+      </c>
+      <c r="L324" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>12</v>
+      </c>
+      <c r="M324" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>80</v>
+      </c>
+      <c r="N324" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>39</v>
+      </c>
+      <c r="O324" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>00</v>
+      </c>
+      <c r="P324" s="2">
+        <f t="shared" si="62"/>
+        <v>21.52</v>
+      </c>
+      <c r="Q324" s="2">
+        <f t="shared" ref="Q324:Q335" si="64">((((O324/60)+N324)/60)+M324)*IF(D324="W",-1, 1)</f>
+        <v>-80.650000000000006</v>
+      </c>
+      <c r="R324" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="325" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A325" s="1">
+        <v>324</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C325" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D325" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E325" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="F325" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="G325" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H325" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I325" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="J325" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K325" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>24</v>
+      </c>
+      <c r="L325" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>36</v>
+      </c>
+      <c r="M325" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>, 82</v>
+      </c>
+      <c r="N325" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>19</v>
+      </c>
+      <c r="O325" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>12</v>
+      </c>
+      <c r="P325" s="2">
+        <f t="shared" si="62"/>
+        <v>21.41</v>
+      </c>
+      <c r="Q325" s="2" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="R325" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="326" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A326" s="1">
+        <v>325</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C326" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D326" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E326" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F326" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="G326" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H326" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I326" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="J326" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K326" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>10</v>
+      </c>
+      <c r="L326" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>48</v>
+      </c>
+      <c r="M326" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>84</v>
+      </c>
+      <c r="N326" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>51</v>
+      </c>
+      <c r="O326" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>36</v>
+      </c>
+      <c r="P326" s="2">
+        <f t="shared" si="62"/>
+        <v>21.18</v>
+      </c>
+      <c r="Q326" s="2">
+        <f t="shared" si="64"/>
+        <v>-84.86</v>
+      </c>
+      <c r="R326" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="327" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A327" s="1">
+        <v>326</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C327" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D327" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E327" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="F327" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="G327" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H327" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I327" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="J327" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K327" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>00</v>
+      </c>
+      <c r="L327" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>00</v>
+      </c>
+      <c r="M327" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>84</v>
+      </c>
+      <c r="N327" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>53</v>
+      </c>
+      <c r="O327" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>24</v>
+      </c>
+      <c r="P327" s="2">
+        <f t="shared" si="62"/>
+        <v>20</v>
+      </c>
+      <c r="Q327" s="2">
+        <f t="shared" si="64"/>
+        <v>-84.89</v>
+      </c>
+      <c r="R327" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="328" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A328" s="1">
+        <v>327</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C328" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D328" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E328" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F328" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="G328" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H328" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I328" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="J328" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K328" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>16</v>
+      </c>
+      <c r="L328" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>12</v>
+      </c>
+      <c r="M328" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N328" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>25</v>
+      </c>
+      <c r="O328" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>12</v>
+      </c>
+      <c r="P328" s="2">
+        <f t="shared" si="62"/>
+        <v>19.27</v>
+      </c>
+      <c r="Q328" s="2">
+        <f t="shared" si="64"/>
+        <v>-82.42</v>
+      </c>
+      <c r="R328" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="329" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A329" s="1">
+        <v>328</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C329" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D329" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E329" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="F329" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="G329" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H329" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I329" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="J329" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K329" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>10</v>
+      </c>
+      <c r="L329" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>12</v>
+      </c>
+      <c r="M329" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>79</v>
+      </c>
+      <c r="N329" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>54</v>
+      </c>
+      <c r="O329" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>00</v>
+      </c>
+      <c r="P329" s="2">
+        <f t="shared" si="62"/>
+        <v>20.170000000000002</v>
+      </c>
+      <c r="Q329" s="2">
+        <f t="shared" si="64"/>
+        <v>-79.900000000000006</v>
+      </c>
+      <c r="R329" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="330" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A330" s="1">
+        <v>329</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C330" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D330" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E330" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="F330" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="G330" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H330" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I330" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="J330" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K330" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>34</v>
+      </c>
+      <c r="L330" s="1" t="e">
+        <f t="shared" si="58"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M330" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>83</v>
+      </c>
+      <c r="N330" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>31</v>
+      </c>
+      <c r="O330" s="1" t="e">
+        <f t="shared" si="61"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P330" s="2" t="e">
+        <f t="shared" si="62"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q330" s="2" t="e">
+        <f t="shared" si="64"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="R330" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="331" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A331" s="1">
+        <v>330</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C331" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D331" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E331" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="F331" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="G331" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="H331" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I331" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J331" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K331" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>41</v>
+      </c>
+      <c r="L331" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>54</v>
+      </c>
+      <c r="M331" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N331" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>27</v>
+      </c>
+      <c r="O331" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>43</v>
+      </c>
+      <c r="P331" s="2">
+        <f t="shared" si="62"/>
+        <v>19.698333333333334</v>
+      </c>
+      <c r="Q331" s="2">
+        <f t="shared" si="64"/>
+        <v>-87.461944444444441</v>
+      </c>
+      <c r="R331" s="16" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="332" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A332" s="1">
+        <v>331</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C332" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D332" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E332" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="F332" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="G332" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="H332" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I332" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J332" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K332" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>43</v>
+      </c>
+      <c r="L332" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>35</v>
+      </c>
+      <c r="M332" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N332" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>25</v>
+      </c>
+      <c r="O332" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>06</v>
+      </c>
+      <c r="P332" s="2">
+        <f t="shared" si="62"/>
+        <v>19.726388888888888</v>
+      </c>
+      <c r="Q332" s="2">
+        <f t="shared" si="64"/>
+        <v>-87.418333333333337</v>
+      </c>
+      <c r="R332" s="16" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="333" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A333" s="1">
+        <v>332</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C333" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D333" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E333" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="F333" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="G333" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="H333" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I333" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J333" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K333" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L333" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>04</v>
+      </c>
+      <c r="M333" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N333" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>25</v>
+      </c>
+      <c r="O333" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>23</v>
+      </c>
+      <c r="P333" s="2">
+        <f t="shared" si="62"/>
+        <v>19.734444444444446</v>
+      </c>
+      <c r="Q333" s="2">
+        <f t="shared" si="64"/>
+        <v>-87.42305555555555</v>
+      </c>
+      <c r="R333" s="16" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="334" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A334" s="1">
+        <v>333</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C334" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D334" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E334" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="F334" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="G334" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="H334" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I334" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J334" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K334" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>46</v>
+      </c>
+      <c r="L334" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>33</v>
+      </c>
+      <c r="M334" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N334" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>28</v>
+      </c>
+      <c r="O334" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>37</v>
+      </c>
+      <c r="P334" s="2">
+        <f t="shared" si="62"/>
+        <v>19.775833333333335</v>
+      </c>
+      <c r="Q334" s="2">
+        <f t="shared" si="64"/>
+        <v>-87.476944444444442</v>
+      </c>
+      <c r="R334" s="16" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="335" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A335" s="1">
+        <v>334</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C335" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D335" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E335" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="F335" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="G335" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="H335" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I335" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J335" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K335" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>38</v>
+      </c>
+      <c r="L335" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>59</v>
+      </c>
+      <c r="M335" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N335" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>27</v>
+      </c>
+      <c r="O335" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>21</v>
+      </c>
+      <c r="P335" s="2">
+        <f t="shared" si="62"/>
+        <v>19.649722222222223</v>
+      </c>
+      <c r="Q335" s="2">
+        <f t="shared" si="64"/>
+        <v>-87.455833333333331</v>
+      </c>
+      <c r="R335" s="16" t="s">
+        <v>484</v>
+      </c>
     </row>
     <row r="336" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="P336" s="2"/>
-      <c r="Q336" s="2"/>
-    </row>
-    <row r="337" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P337" s="2"/>
-      <c r="Q337" s="2"/>
-    </row>
-    <row r="338" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P338" s="2"/>
-      <c r="Q338" s="2"/>
-    </row>
-    <row r="339" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P339" s="2"/>
-      <c r="Q339" s="2"/>
-    </row>
-    <row r="340" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P340" s="2"/>
-      <c r="Q340" s="2"/>
-    </row>
-    <row r="341" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P341" s="2"/>
-      <c r="Q341" s="2"/>
-    </row>
-    <row r="342" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P342" s="2"/>
-      <c r="Q342" s="2"/>
-    </row>
-    <row r="343" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P343" s="2"/>
-      <c r="Q343" s="2"/>
-    </row>
-    <row r="344" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P344" s="2"/>
-      <c r="Q344" s="2"/>
-    </row>
-    <row r="345" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P345" s="2"/>
-      <c r="Q345" s="2"/>
-    </row>
-    <row r="346" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P346" s="2"/>
-      <c r="Q346" s="2"/>
-    </row>
-    <row r="347" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P347" s="2"/>
-      <c r="Q347" s="2"/>
-    </row>
-    <row r="348" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P348" s="2"/>
-      <c r="Q348" s="2"/>
-    </row>
-    <row r="349" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P349" s="2"/>
-      <c r="Q349" s="2"/>
-    </row>
-    <row r="350" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P350" s="2"/>
-      <c r="Q350" s="2"/>
-    </row>
-    <row r="351" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P351" s="2"/>
-      <c r="Q351" s="2"/>
-    </row>
-    <row r="352" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P352" s="2"/>
-      <c r="Q352" s="2"/>
-    </row>
-    <row r="353" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P353" s="2"/>
-      <c r="Q353" s="2"/>
-    </row>
-    <row r="354" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P354" s="2"/>
-      <c r="Q354" s="2"/>
-    </row>
-    <row r="355" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P355" s="2"/>
-      <c r="Q355" s="2"/>
-    </row>
-    <row r="356" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P356" s="2"/>
-      <c r="Q356" s="2"/>
-    </row>
-    <row r="357" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P357" s="2"/>
-      <c r="Q357" s="2"/>
-    </row>
-    <row r="358" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P358" s="2"/>
-      <c r="Q358" s="2"/>
-    </row>
-    <row r="359" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P359" s="2"/>
-      <c r="Q359" s="2"/>
-    </row>
-    <row r="360" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P360" s="2"/>
-      <c r="Q360" s="2"/>
-    </row>
-    <row r="361" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P361" s="2"/>
-      <c r="Q361" s="2"/>
-    </row>
-    <row r="362" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P362" s="2"/>
-      <c r="Q362" s="2"/>
-    </row>
-    <row r="363" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P363" s="2"/>
-      <c r="Q363" s="2"/>
-    </row>
-    <row r="364" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P364" s="2"/>
-      <c r="Q364" s="2"/>
-    </row>
-    <row r="365" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P365" s="2"/>
-      <c r="Q365" s="2"/>
-    </row>
-    <row r="366" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P366" s="2"/>
-      <c r="Q366" s="2"/>
-    </row>
-    <row r="367" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P367" s="2"/>
-      <c r="Q367" s="2"/>
-    </row>
-    <row r="368" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P368" s="2"/>
-      <c r="Q368" s="2"/>
-    </row>
-    <row r="369" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P369" s="2"/>
-      <c r="Q369" s="2"/>
-    </row>
-    <row r="370" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P370" s="2"/>
-      <c r="Q370" s="2"/>
-    </row>
-    <row r="371" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P371" s="2"/>
-      <c r="Q371" s="2"/>
-    </row>
-    <row r="372" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P372" s="2"/>
-      <c r="Q372" s="2"/>
-    </row>
-    <row r="373" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P373" s="2"/>
-      <c r="Q373" s="2"/>
-    </row>
-    <row r="374" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P374" s="2"/>
-      <c r="Q374" s="2"/>
-    </row>
-    <row r="375" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P375" s="2"/>
-      <c r="Q375" s="2"/>
-    </row>
-    <row r="376" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P376" s="2"/>
-      <c r="Q376" s="2"/>
-    </row>
-    <row r="377" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P377" s="2"/>
-      <c r="Q377" s="2"/>
-    </row>
-    <row r="378" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P378" s="2"/>
-      <c r="Q378" s="2"/>
-    </row>
-    <row r="379" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="P379" s="2"/>
-      <c r="Q379" s="2"/>
-    </row>
-    <row r="380" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B380" s="7"/>
-      <c r="G380" s="7"/>
-      <c r="H380" s="7"/>
-      <c r="P380" s="2"/>
-      <c r="Q380" s="2"/>
-    </row>
-    <row r="381" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B381" s="18"/>
-      <c r="E381" s="18"/>
-      <c r="F381" s="18"/>
-      <c r="G381" s="7"/>
-      <c r="H381" s="7"/>
-      <c r="I381" s="10"/>
-      <c r="P381" s="2"/>
-      <c r="Q381" s="2"/>
-    </row>
-    <row r="382" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B382" s="18"/>
-      <c r="E382" s="18"/>
-      <c r="F382" s="18"/>
-      <c r="G382" s="7"/>
-      <c r="H382" s="7"/>
-      <c r="I382" s="10"/>
-      <c r="P382" s="2"/>
-      <c r="Q382" s="2"/>
-    </row>
-    <row r="383" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B383" s="18"/>
-      <c r="E383" s="18"/>
-      <c r="F383" s="18"/>
-      <c r="G383" s="7"/>
-      <c r="H383" s="7"/>
-      <c r="I383" s="10"/>
-      <c r="P383" s="2"/>
-      <c r="Q383" s="2"/>
-    </row>
-    <row r="384" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B384" s="18"/>
-      <c r="E384" s="18"/>
-      <c r="F384" s="18"/>
-      <c r="G384" s="7"/>
-      <c r="H384" s="7"/>
-      <c r="I384" s="10"/>
-      <c r="P384" s="2"/>
-      <c r="Q384" s="2"/>
-    </row>
-    <row r="385" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B385" s="18"/>
-      <c r="E385" s="18"/>
-      <c r="F385" s="18"/>
-      <c r="G385" s="7"/>
-      <c r="H385" s="7"/>
-      <c r="I385" s="10"/>
-      <c r="P385" s="2"/>
-      <c r="Q385" s="2"/>
-    </row>
-    <row r="386" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B386" s="18"/>
-      <c r="E386" s="18"/>
-      <c r="F386" s="18"/>
-      <c r="G386" s="7"/>
-      <c r="H386" s="7"/>
-      <c r="I386" s="10"/>
-      <c r="P386" s="2"/>
-      <c r="Q386" s="2"/>
-    </row>
-    <row r="387" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B387" s="18"/>
-      <c r="E387" s="10"/>
-      <c r="F387" s="10"/>
-      <c r="G387" s="7"/>
-      <c r="H387" s="7"/>
-      <c r="I387" s="10"/>
-      <c r="P387" s="2"/>
-      <c r="Q387" s="2"/>
-    </row>
-    <row r="388" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="A336" s="1">
+        <v>335</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C336" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D336" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E336" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="F336" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="G336" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="H336" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I336" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J336" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K336" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>38</v>
+      </c>
+      <c r="L336" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>36</v>
+      </c>
+      <c r="M336" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N336" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>27</v>
+      </c>
+      <c r="O336" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>36</v>
+      </c>
+      <c r="P336" s="2">
+        <f t="shared" si="62"/>
+        <v>19.643333333333334</v>
+      </c>
+      <c r="Q336" s="2">
+        <f t="shared" ref="Q336:Q384" si="65">((((O336/60)+N336)/60)+M336)*IF(D337="W",-1, 1)</f>
+        <v>-87.46</v>
+      </c>
+      <c r="R336" s="16" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="337" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A337" s="1">
+        <v>336</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C337" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D337" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E337" s="7" t="s">
+        <v>535</v>
+      </c>
+      <c r="F337" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="G337" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H337" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I337" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J337" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>09</v>
+      </c>
+      <c r="K337" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L337" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>15</v>
+      </c>
+      <c r="M337" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N337" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>49</v>
+      </c>
+      <c r="O337" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>28</v>
+      </c>
+      <c r="P337" s="2">
+        <f t="shared" si="62"/>
+        <v>9.7375000000000007</v>
+      </c>
+      <c r="Q337" s="2">
+        <f t="shared" si="65"/>
+        <v>-82.824444444444438</v>
+      </c>
+      <c r="R337" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="338" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A338" s="1">
+        <v>337</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C338" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D338" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E338" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="F338" s="7" t="s">
+        <v>540</v>
+      </c>
+      <c r="G338" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H338" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I338" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J338" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>09</v>
+      </c>
+      <c r="K338" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L338" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>24</v>
+      </c>
+      <c r="M338" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N338" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>49</v>
+      </c>
+      <c r="O338" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>19</v>
+      </c>
+      <c r="P338" s="2">
+        <f t="shared" si="62"/>
+        <v>9.74</v>
+      </c>
+      <c r="Q338" s="2">
+        <f t="shared" si="65"/>
+        <v>-82.821944444444441</v>
+      </c>
+      <c r="R338" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="339" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A339" s="1">
+        <v>338</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C339" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D339" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E339" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="F339" s="7" t="s">
+        <v>542</v>
+      </c>
+      <c r="G339" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H339" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I339" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J339" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>09</v>
+      </c>
+      <c r="K339" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L339" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>48</v>
+      </c>
+      <c r="M339" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N339" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>49</v>
+      </c>
+      <c r="O339" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>08</v>
+      </c>
+      <c r="P339" s="2">
+        <f t="shared" si="62"/>
+        <v>9.7466666666666661</v>
+      </c>
+      <c r="Q339" s="2">
+        <f t="shared" si="65"/>
+        <v>-82.818888888888893</v>
+      </c>
+      <c r="R339" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="340" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A340" s="1">
+        <v>339</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C340" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D340" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E340" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="F340" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="G340" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H340" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I340" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J340" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>09</v>
+      </c>
+      <c r="K340" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L340" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>36</v>
+      </c>
+      <c r="M340" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N340" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>48</v>
+      </c>
+      <c r="O340" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>23</v>
+      </c>
+      <c r="P340" s="2">
+        <f t="shared" si="62"/>
+        <v>9.7433333333333341</v>
+      </c>
+      <c r="Q340" s="2">
+        <f t="shared" si="65"/>
+        <v>-82.80638888888889</v>
+      </c>
+      <c r="R340" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="341" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A341" s="1">
+        <v>340</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C341" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D341" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E341" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="F341" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="G341" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H341" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I341" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J341" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>09</v>
+      </c>
+      <c r="K341" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L341" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>29</v>
+      </c>
+      <c r="M341" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N341" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>48</v>
+      </c>
+      <c r="O341" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>32</v>
+      </c>
+      <c r="P341" s="2">
+        <f t="shared" si="62"/>
+        <v>9.7413888888888884</v>
+      </c>
+      <c r="Q341" s="2">
+        <f t="shared" si="65"/>
+        <v>-82.808888888888887</v>
+      </c>
+      <c r="R341" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="342" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A342" s="1">
+        <v>341</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C342" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D342" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E342" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="F342" s="7" t="s">
+        <v>548</v>
+      </c>
+      <c r="G342" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H342" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I342" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J342" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>09</v>
+      </c>
+      <c r="K342" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>44</v>
+      </c>
+      <c r="L342" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>16</v>
+      </c>
+      <c r="M342" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>82</v>
+      </c>
+      <c r="N342" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>48</v>
+      </c>
+      <c r="O342" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>30</v>
+      </c>
+      <c r="P342" s="2">
+        <f t="shared" si="62"/>
+        <v>9.7377777777777776</v>
+      </c>
+      <c r="Q342" s="2">
+        <f t="shared" si="65"/>
+        <v>-82.808333333333337</v>
+      </c>
+      <c r="R342" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="343" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A343" s="1">
+        <v>342</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C343" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D343" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E343" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="F343" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="G343" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H343" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I343" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J343" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K343" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>05</v>
+      </c>
+      <c r="L343" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>44</v>
+      </c>
+      <c r="M343" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N343" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>23</v>
+      </c>
+      <c r="O343" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>22</v>
+      </c>
+      <c r="P343" s="2">
+        <f t="shared" si="62"/>
+        <v>19.095555555555556</v>
+      </c>
+      <c r="Q343" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.38944444444445</v>
+      </c>
+      <c r="R343" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="344" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A344" s="1">
+        <v>343</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C344" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D344" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E344" s="20" t="s">
+        <v>585</v>
+      </c>
+      <c r="F344" s="20" t="s">
+        <v>602</v>
+      </c>
+      <c r="G344" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H344" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I344" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J344" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K344" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>01</v>
+      </c>
+      <c r="L344" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>25</v>
+      </c>
+      <c r="M344" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N344" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>11</v>
+      </c>
+      <c r="O344" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>20</v>
+      </c>
+      <c r="P344" s="2">
+        <f t="shared" si="62"/>
+        <v>19.023611111111112</v>
+      </c>
+      <c r="Q344" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.188888888888883</v>
+      </c>
+      <c r="R344" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="345" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A345" s="1">
+        <v>344</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C345" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D345" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E345" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="F345" s="20" t="s">
+        <v>601</v>
+      </c>
+      <c r="G345" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H345" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I345" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J345" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>18</v>
+      </c>
+      <c r="K345" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>57</v>
+      </c>
+      <c r="L345" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>22</v>
+      </c>
+      <c r="M345" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N345" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>57</v>
+      </c>
+      <c r="O345" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>43</v>
+      </c>
+      <c r="P345" s="2">
+        <f t="shared" si="62"/>
+        <v>18.95611111111111</v>
+      </c>
+      <c r="Q345" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.961944444444441</v>
+      </c>
+      <c r="R345" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="346" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A346" s="1">
+        <v>345</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C346" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D346" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E346" s="20" t="s">
+        <v>587</v>
+      </c>
+      <c r="F346" s="20" t="s">
+        <v>600</v>
+      </c>
+      <c r="G346" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H346" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I346" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J346" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>18</v>
+      </c>
+      <c r="K346" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>51</v>
+      </c>
+      <c r="L346" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>45</v>
+      </c>
+      <c r="M346" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N346" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>42</v>
+      </c>
+      <c r="O346" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>33</v>
+      </c>
+      <c r="P346" s="2">
+        <f t="shared" si="62"/>
+        <v>18.862500000000001</v>
+      </c>
+      <c r="Q346" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.709166666666661</v>
+      </c>
+      <c r="R346" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="347" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A347" s="1">
+        <v>346</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C347" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D347" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E347" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="F347" s="20" t="s">
+        <v>599</v>
+      </c>
+      <c r="G347" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H347" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I347" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J347" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K347" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>26</v>
+      </c>
+      <c r="L347" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>27</v>
+      </c>
+      <c r="M347" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N347" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>14</v>
+      </c>
+      <c r="O347" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>30</v>
+      </c>
+      <c r="P347" s="2">
+        <f t="shared" si="62"/>
+        <v>19.440833333333334</v>
+      </c>
+      <c r="Q347" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.24166666666666</v>
+      </c>
+      <c r="R347" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="348" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A348" s="1">
+        <v>347</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C348" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D348" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E348" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="F348" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G348" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H348" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I348" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J348" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K348" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>24</v>
+      </c>
+      <c r="L348" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>32</v>
+      </c>
+      <c r="M348" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N348" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>02</v>
+      </c>
+      <c r="O348" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>45</v>
+      </c>
+      <c r="P348" s="2">
+        <f t="shared" si="62"/>
+        <v>19.408888888888889</v>
+      </c>
+      <c r="Q348" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.045833333333334</v>
+      </c>
+      <c r="R348" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="349" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A349" s="1">
+        <v>348</v>
+      </c>
+      <c r="B349" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C349" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D349" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E349" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="F349" s="20" t="s">
+        <v>597</v>
+      </c>
+      <c r="G349" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H349" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I349" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J349" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K349" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>22</v>
+      </c>
+      <c r="L349" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>01</v>
+      </c>
+      <c r="M349" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N349" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>51</v>
+      </c>
+      <c r="O349" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>20</v>
+      </c>
+      <c r="P349" s="2">
+        <f t="shared" si="62"/>
+        <v>19.366944444444446</v>
+      </c>
+      <c r="Q349" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.855555555555554</v>
+      </c>
+      <c r="R349" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="350" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A350" s="1">
+        <v>349</v>
+      </c>
+      <c r="B350" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C350" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D350" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E350" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="F350" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="G350" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H350" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I350" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J350" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K350" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>18</v>
+      </c>
+      <c r="L350" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>32</v>
+      </c>
+      <c r="M350" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N350" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>37</v>
+      </c>
+      <c r="O350" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>24</v>
+      </c>
+      <c r="P350" s="2">
+        <f t="shared" si="62"/>
+        <v>19.308888888888887</v>
+      </c>
+      <c r="Q350" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.623333333333335</v>
+      </c>
+      <c r="R350" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="351" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A351" s="1">
+        <v>350</v>
+      </c>
+      <c r="B351" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C351" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D351" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E351" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="F351" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="G351" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H351" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I351" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J351" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K351" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>14</v>
+      </c>
+      <c r="L351" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>28</v>
+      </c>
+      <c r="M351" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N351" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>25</v>
+      </c>
+      <c r="O351" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>23</v>
+      </c>
+      <c r="P351" s="2">
+        <f t="shared" si="62"/>
+        <v>19.24111111111111</v>
+      </c>
+      <c r="Q351" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.42305555555555</v>
+      </c>
+      <c r="R351" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="352" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A352" s="1">
+        <v>351</v>
+      </c>
+      <c r="B352" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C352" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D352" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E352" s="20" t="s">
+        <v>593</v>
+      </c>
+      <c r="F352" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="G352" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H352" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I352" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J352" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K352" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>11</v>
+      </c>
+      <c r="L352" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>54</v>
+      </c>
+      <c r="M352" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N352" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>15</v>
+      </c>
+      <c r="O352" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>33</v>
+      </c>
+      <c r="P352" s="2">
+        <f t="shared" si="62"/>
+        <v>19.198333333333334</v>
+      </c>
+      <c r="Q352" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.259166666666673</v>
+      </c>
+      <c r="R352" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="353" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A353" s="1">
+        <v>352</v>
+      </c>
+      <c r="B353" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C353" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D353" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E353" s="20" t="s">
+        <v>605</v>
+      </c>
+      <c r="F353" s="20" t="s">
+        <v>631</v>
+      </c>
+      <c r="G353" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H353" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I353" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J353" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K353" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>49</v>
+      </c>
+      <c r="L353" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>18</v>
+      </c>
+      <c r="M353" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N353" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>24</v>
+      </c>
+      <c r="O353" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>21</v>
+      </c>
+      <c r="P353" s="2">
+        <f t="shared" si="62"/>
+        <v>19.821666666666665</v>
+      </c>
+      <c r="Q353" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.405833333333334</v>
+      </c>
+      <c r="R353" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="354" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A354" s="1">
+        <v>353</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C354" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D354" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E354" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="F354" s="20" t="s">
+        <v>630</v>
+      </c>
+      <c r="G354" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H354" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I354" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J354" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K354" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>45</v>
+      </c>
+      <c r="L354" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>51</v>
+      </c>
+      <c r="M354" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N354" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>12</v>
+      </c>
+      <c r="O354" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>24</v>
+      </c>
+      <c r="P354" s="2">
+        <f t="shared" si="62"/>
+        <v>19.764166666666668</v>
+      </c>
+      <c r="Q354" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.206666666666663</v>
+      </c>
+      <c r="R354" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="355" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A355" s="1">
+        <v>354</v>
+      </c>
+      <c r="B355" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C355" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D355" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E355" s="20" t="s">
+        <v>668</v>
+      </c>
+      <c r="F355" s="20" t="s">
+        <v>629</v>
+      </c>
+      <c r="G355" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H355" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I355" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J355" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K355" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>48</v>
+      </c>
+      <c r="L355" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>21</v>
+      </c>
+      <c r="M355" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N355" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>59</v>
+      </c>
+      <c r="O355" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>06</v>
+      </c>
+      <c r="P355" s="2">
+        <f t="shared" si="62"/>
+        <v>19.805833333333332</v>
+      </c>
+      <c r="Q355" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.984999999999999</v>
+      </c>
+      <c r="R355" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="356" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A356" s="1">
+        <v>355</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C356" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D356" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E356" s="20" t="s">
+        <v>607</v>
+      </c>
+      <c r="F356" s="20" t="s">
+        <v>628</v>
+      </c>
+      <c r="G356" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H356" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I356" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J356" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K356" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>59</v>
+      </c>
+      <c r="L356" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>09</v>
+      </c>
+      <c r="M356" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N356" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>26</v>
+      </c>
+      <c r="O356" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>19</v>
+      </c>
+      <c r="P356" s="2">
+        <f t="shared" si="62"/>
+        <v>19.985833333333332</v>
+      </c>
+      <c r="Q356" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.438611111111115</v>
+      </c>
+      <c r="R356" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="357" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A357" s="1">
+        <v>356</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C357" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D357" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E357" s="20" t="s">
+        <v>608</v>
+      </c>
+      <c r="F357" s="20" t="s">
+        <v>627</v>
+      </c>
+      <c r="G357" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H357" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I357" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J357" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K357" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>00</v>
+      </c>
+      <c r="L357" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>22</v>
+      </c>
+      <c r="M357" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N357" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>13</v>
+      </c>
+      <c r="O357" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>16</v>
+      </c>
+      <c r="P357" s="2">
+        <f t="shared" si="62"/>
+        <v>20.00611111111111</v>
+      </c>
+      <c r="Q357" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.221111111111114</v>
+      </c>
+      <c r="R357" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="358" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A358" s="1">
+        <v>357</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C358" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D358" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E358" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="F358" s="20" t="s">
+        <v>626</v>
+      </c>
+      <c r="G358" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H358" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I358" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J358" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>19</v>
+      </c>
+      <c r="K358" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>58</v>
+      </c>
+      <c r="L358" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>01</v>
+      </c>
+      <c r="M358" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N358" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>07</v>
+      </c>
+      <c r="O358" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>18</v>
+      </c>
+      <c r="P358" s="2">
+        <f t="shared" si="62"/>
+        <v>19.966944444444444</v>
+      </c>
+      <c r="Q358" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.12166666666667</v>
+      </c>
+      <c r="R358" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="359" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A359" s="1">
+        <v>358</v>
+      </c>
+      <c r="B359" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C359" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D359" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E359" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="F359" s="20" t="s">
+        <v>625</v>
+      </c>
+      <c r="G359" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H359" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I359" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J359" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K359" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>00</v>
+      </c>
+      <c r="L359" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>33</v>
+      </c>
+      <c r="M359" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N359" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>58</v>
+      </c>
+      <c r="O359" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>42</v>
+      </c>
+      <c r="P359" s="2">
+        <f t="shared" si="62"/>
+        <v>20.009166666666665</v>
+      </c>
+      <c r="Q359" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.978333333333339</v>
+      </c>
+      <c r="R359" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="360" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A360" s="1">
+        <v>359</v>
+      </c>
+      <c r="B360" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C360" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D360" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E360" s="20" t="s">
+        <v>611</v>
+      </c>
+      <c r="F360" s="20" t="s">
+        <v>624</v>
+      </c>
+      <c r="G360" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H360" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I360" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J360" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K360" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>02</v>
+      </c>
+      <c r="L360" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>16</v>
+      </c>
+      <c r="M360" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N360" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>41</v>
+      </c>
+      <c r="O360" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>19</v>
+      </c>
+      <c r="P360" s="2">
+        <f t="shared" si="62"/>
+        <v>20.037777777777777</v>
+      </c>
+      <c r="Q360" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.688611111111115</v>
+      </c>
+      <c r="R360" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="361" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A361" s="1">
+        <v>360</v>
+      </c>
+      <c r="B361" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C361" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D361" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E361" s="20" t="s">
+        <v>612</v>
+      </c>
+      <c r="F361" s="20" t="s">
+        <v>623</v>
+      </c>
+      <c r="G361" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H361" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I361" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J361" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K361" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>01</v>
+      </c>
+      <c r="L361" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>15</v>
+      </c>
+      <c r="M361" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N361" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>30</v>
+      </c>
+      <c r="O361" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>41</v>
+      </c>
+      <c r="P361" s="2">
+        <f t="shared" si="62"/>
+        <v>20.020833333333332</v>
+      </c>
+      <c r="Q361" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.511388888888888</v>
+      </c>
+      <c r="R361" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="362" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A362" s="1">
+        <v>361</v>
+      </c>
+      <c r="B362" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C362" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D362" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E362" s="20" t="s">
+        <v>613</v>
+      </c>
+      <c r="F362" s="20" t="s">
+        <v>622</v>
+      </c>
+      <c r="G362" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H362" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I362" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J362" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K362" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>14</v>
+      </c>
+      <c r="L362" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>26</v>
+      </c>
+      <c r="M362" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N362" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>16</v>
+      </c>
+      <c r="O362" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>43</v>
+      </c>
+      <c r="P362" s="2">
+        <f t="shared" si="62"/>
+        <v>20.240555555555556</v>
+      </c>
+      <c r="Q362" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.278611111111104</v>
+      </c>
+      <c r="R362" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="363" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A363" s="1">
+        <v>362</v>
+      </c>
+      <c r="B363" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C363" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D363" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E363" s="20" t="s">
+        <v>614</v>
+      </c>
+      <c r="F363" s="20" t="s">
+        <v>621</v>
+      </c>
+      <c r="G363" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H363" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I363" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J363" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K363" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>13</v>
+      </c>
+      <c r="L363" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>06</v>
+      </c>
+      <c r="M363" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>87</v>
+      </c>
+      <c r="N363" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>08</v>
+      </c>
+      <c r="O363" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>06</v>
+      </c>
+      <c r="P363" s="2">
+        <f t="shared" si="62"/>
+        <v>20.218333333333334</v>
+      </c>
+      <c r="Q363" s="2">
+        <f t="shared" si="65"/>
+        <v>-87.135000000000005</v>
+      </c>
+      <c r="R363" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="364" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A364" s="1">
+        <v>363</v>
+      </c>
+      <c r="B364" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C364" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D364" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E364" s="20" t="s">
+        <v>615</v>
+      </c>
+      <c r="F364" s="20" t="s">
+        <v>620</v>
+      </c>
+      <c r="G364" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H364" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I364" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J364" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K364" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>08</v>
+      </c>
+      <c r="L364" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>38</v>
+      </c>
+      <c r="M364" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N364" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>59</v>
+      </c>
+      <c r="O364" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>43</v>
+      </c>
+      <c r="P364" s="2">
+        <f t="shared" si="62"/>
+        <v>20.143888888888888</v>
+      </c>
+      <c r="Q364" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.995277777777773</v>
+      </c>
+      <c r="R364" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="365" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A365" s="1">
+        <v>364</v>
+      </c>
+      <c r="B365" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C365" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D365" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E365" s="20" t="s">
+        <v>616</v>
+      </c>
+      <c r="F365" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="G365" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H365" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I365" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J365" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K365" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>12</v>
+      </c>
+      <c r="L365" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>54</v>
+      </c>
+      <c r="M365" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N365" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>50</v>
+      </c>
+      <c r="O365" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>07</v>
+      </c>
+      <c r="P365" s="2">
+        <f t="shared" si="62"/>
+        <v>20.215</v>
+      </c>
+      <c r="Q365" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.835277777777776</v>
+      </c>
+      <c r="R365" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="366" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A366" s="1">
+        <v>365</v>
+      </c>
+      <c r="B366" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C366" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D366" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E366" s="20" t="s">
+        <v>617</v>
+      </c>
+      <c r="F366" s="20" t="s">
+        <v>618</v>
+      </c>
+      <c r="G366" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H366" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I366" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J366" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K366" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>13</v>
+      </c>
+      <c r="L366" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>16</v>
+      </c>
+      <c r="M366" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N366" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>37</v>
+      </c>
+      <c r="O366" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>47</v>
+      </c>
+      <c r="P366" s="2">
+        <f t="shared" si="62"/>
+        <v>20.22111111111111</v>
+      </c>
+      <c r="Q366" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.629722222222227</v>
+      </c>
+      <c r="R366" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="367" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A367" s="1">
+        <v>366</v>
+      </c>
+      <c r="B367" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C367" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D367" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E367" s="20" t="s">
+        <v>632</v>
+      </c>
+      <c r="F367" s="20" t="s">
+        <v>667</v>
+      </c>
+      <c r="G367" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H367" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I367" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J367" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K367" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>41</v>
+      </c>
+      <c r="L367" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>46</v>
+      </c>
+      <c r="M367" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N367" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>52</v>
+      </c>
+      <c r="O367" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>49</v>
+      </c>
+      <c r="P367" s="2">
+        <f t="shared" si="62"/>
+        <v>20.696111111111112</v>
+      </c>
+      <c r="Q367" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.880277777777778</v>
+      </c>
+      <c r="R367" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="368" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A368" s="1">
+        <v>367</v>
+      </c>
+      <c r="B368" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C368" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D368" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E368" s="20" t="s">
+        <v>633</v>
+      </c>
+      <c r="F368" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="G368" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H368" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I368" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J368" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K368" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>32</v>
+      </c>
+      <c r="L368" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>40</v>
+      </c>
+      <c r="M368" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N368" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>29</v>
+      </c>
+      <c r="O368" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>49</v>
+      </c>
+      <c r="P368" s="2">
+        <f t="shared" si="62"/>
+        <v>20.544444444444444</v>
+      </c>
+      <c r="Q368" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.496944444444438</v>
+      </c>
+      <c r="R368" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="369" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A369" s="1">
+        <v>368</v>
+      </c>
+      <c r="B369" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C369" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D369" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E369" s="20" t="s">
+        <v>634</v>
+      </c>
+      <c r="F369" s="20" t="s">
+        <v>665</v>
+      </c>
+      <c r="G369" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H369" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I369" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J369" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K369" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>30</v>
+      </c>
+      <c r="L369" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>05</v>
+      </c>
+      <c r="M369" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N369" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>20</v>
+      </c>
+      <c r="O369" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>32</v>
+      </c>
+      <c r="P369" s="2">
+        <f t="shared" si="62"/>
+        <v>20.50138888888889</v>
+      </c>
+      <c r="Q369" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.342222222222219</v>
+      </c>
+      <c r="R369" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="370" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A370" s="1">
+        <v>369</v>
+      </c>
+      <c r="B370" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C370" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D370" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E370" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="F370" s="20" t="s">
+        <v>664</v>
+      </c>
+      <c r="G370" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H370" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I370" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J370" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K370" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>31</v>
+      </c>
+      <c r="L370" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>51</v>
+      </c>
+      <c r="M370" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>85</v>
+      </c>
+      <c r="N370" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>59</v>
+      </c>
+      <c r="O370" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>29</v>
+      </c>
+      <c r="P370" s="2">
+        <f t="shared" si="62"/>
+        <v>20.530833333333334</v>
+      </c>
+      <c r="Q370" s="2">
+        <f t="shared" si="65"/>
+        <v>-85.991388888888892</v>
+      </c>
+      <c r="R370" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="371" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A371" s="1">
+        <v>370</v>
+      </c>
+      <c r="B371" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C371" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D371" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E371" s="20" t="s">
+        <v>636</v>
+      </c>
+      <c r="F371" s="20" t="s">
+        <v>663</v>
+      </c>
+      <c r="G371" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H371" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I371" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J371" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K371" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>47</v>
+      </c>
+      <c r="L371" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>18</v>
+      </c>
+      <c r="M371" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N371" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>45</v>
+      </c>
+      <c r="O371" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>57</v>
+      </c>
+      <c r="P371" s="2">
+        <f t="shared" si="62"/>
+        <v>20.788333333333334</v>
+      </c>
+      <c r="Q371" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.765833333333333</v>
+      </c>
+      <c r="R371" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="372" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A372" s="1">
+        <v>371</v>
+      </c>
+      <c r="B372" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C372" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D372" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E372" s="20" t="s">
+        <v>637</v>
+      </c>
+      <c r="F372" s="20" t="s">
+        <v>662</v>
+      </c>
+      <c r="G372" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H372" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I372" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J372" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K372" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>02</v>
+      </c>
+      <c r="L372" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>26</v>
+      </c>
+      <c r="M372" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N372" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>29</v>
+      </c>
+      <c r="O372" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>47</v>
+      </c>
+      <c r="P372" s="2">
+        <f t="shared" si="62"/>
+        <v>21.040555555555557</v>
+      </c>
+      <c r="Q372" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.496388888888887</v>
+      </c>
+      <c r="R372" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="373" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A373" s="1">
+        <v>372</v>
+      </c>
+      <c r="B373" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C373" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D373" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E373" s="20" t="s">
+        <v>638</v>
+      </c>
+      <c r="F373" s="20" t="s">
+        <v>661</v>
+      </c>
+      <c r="G373" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H373" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I373" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J373" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K373" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>57</v>
+      </c>
+      <c r="L373" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>52</v>
+      </c>
+      <c r="M373" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N373" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>19</v>
+      </c>
+      <c r="O373" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>30</v>
+      </c>
+      <c r="P373" s="2">
+        <f t="shared" si="62"/>
+        <v>20.964444444444446</v>
+      </c>
+      <c r="Q373" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.325000000000003</v>
+      </c>
+      <c r="R373" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="374" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A374" s="1">
+        <v>373</v>
+      </c>
+      <c r="B374" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C374" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D374" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E374" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="F374" s="20" t="s">
+        <v>660</v>
+      </c>
+      <c r="G374" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H374" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I374" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J374" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K374" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>52</v>
+      </c>
+      <c r="L374" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>54</v>
+      </c>
+      <c r="M374" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N374" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>08</v>
+      </c>
+      <c r="O374" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>30</v>
+      </c>
+      <c r="P374" s="2">
+        <f t="shared" si="62"/>
+        <v>20.881666666666668</v>
+      </c>
+      <c r="Q374" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.141666666666666</v>
+      </c>
+      <c r="R374" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="375" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A375" s="1">
+        <v>374</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C375" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D375" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E375" s="20" t="s">
+        <v>640</v>
+      </c>
+      <c r="F375" s="20" t="s">
+        <v>659</v>
+      </c>
+      <c r="G375" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H375" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I375" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J375" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K375" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>50</v>
+      </c>
+      <c r="L375" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>55</v>
+      </c>
+      <c r="M375" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>85</v>
+      </c>
+      <c r="N375" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>53</v>
+      </c>
+      <c r="O375" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>52</v>
+      </c>
+      <c r="P375" s="2">
+        <f t="shared" si="62"/>
+        <v>20.848611111111111</v>
+      </c>
+      <c r="Q375" s="2">
+        <f t="shared" si="65"/>
+        <v>-85.897777777777776</v>
+      </c>
+      <c r="R375" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="376" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A376" s="1">
+        <v>375</v>
+      </c>
+      <c r="B376" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C376" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D376" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E376" s="20" t="s">
+        <v>641</v>
+      </c>
+      <c r="F376" s="20" t="s">
+        <v>658</v>
+      </c>
+      <c r="G376" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H376" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I376" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J376" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>20</v>
+      </c>
+      <c r="K376" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>47</v>
+      </c>
+      <c r="L376" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>16</v>
+      </c>
+      <c r="M376" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>85</v>
+      </c>
+      <c r="N376" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>46</v>
+      </c>
+      <c r="O376" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>28</v>
+      </c>
+      <c r="P376" s="2">
+        <f t="shared" si="62"/>
+        <v>20.787777777777777</v>
+      </c>
+      <c r="Q376" s="2">
+        <f t="shared" si="65"/>
+        <v>-85.774444444444441</v>
+      </c>
+      <c r="R376" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="377" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A377" s="1">
+        <v>376</v>
+      </c>
+      <c r="B377" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C377" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D377" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E377" s="20" t="s">
+        <v>642</v>
+      </c>
+      <c r="F377" s="20" t="s">
+        <v>657</v>
+      </c>
+      <c r="G377" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H377" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I377" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J377" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K377" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>15</v>
+      </c>
+      <c r="L377" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>14</v>
+      </c>
+      <c r="M377" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N377" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>29</v>
+      </c>
+      <c r="O377" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>13</v>
+      </c>
+      <c r="P377" s="2">
+        <f t="shared" si="62"/>
+        <v>21.253888888888888</v>
+      </c>
+      <c r="Q377" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.486944444444447</v>
+      </c>
+      <c r="R377" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="378" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A378" s="1">
+        <v>377</v>
+      </c>
+      <c r="B378" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C378" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D378" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E378" s="20" t="s">
+        <v>643</v>
+      </c>
+      <c r="F378" s="20" t="s">
+        <v>656</v>
+      </c>
+      <c r="G378" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H378" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I378" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J378" s="1" t="str">
+        <f t="shared" si="56"/>
+        <v>21</v>
+      </c>
+      <c r="K378" s="1" t="str">
+        <f t="shared" si="57"/>
+        <v>12</v>
+      </c>
+      <c r="L378" s="1" t="str">
+        <f t="shared" si="58"/>
+        <v>57</v>
+      </c>
+      <c r="M378" s="1" t="str">
+        <f t="shared" si="59"/>
+        <v>86</v>
+      </c>
+      <c r="N378" s="1" t="str">
+        <f t="shared" si="60"/>
+        <v>16</v>
+      </c>
+      <c r="O378" s="1" t="str">
+        <f t="shared" si="61"/>
+        <v>38</v>
+      </c>
+      <c r="P378" s="2">
+        <f t="shared" si="62"/>
+        <v>21.215833333333332</v>
+      </c>
+      <c r="Q378" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.277222222222221</v>
+      </c>
+      <c r="R378" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="379" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A379" s="1">
+        <v>378</v>
+      </c>
+      <c r="B379" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C379" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D379" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E379" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="F379" s="20" t="s">
+        <v>655</v>
+      </c>
+      <c r="G379" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H379" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I379" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J379" s="1" t="str">
+        <f t="shared" ref="J379:J387" si="66">MID(E379,1,FIND("°",E379,1)-1)</f>
+        <v>21</v>
+      </c>
+      <c r="K379" s="1" t="str">
+        <f t="shared" ref="K379:K387" si="67">MID(E379,FIND("°",E379,1)+1,(FIND("′",E379,1)-FIND("°",E379,1))-1)</f>
+        <v>09</v>
+      </c>
+      <c r="L379" s="1" t="str">
+        <f t="shared" ref="L379:L387" si="68">MID(E379,FIND("′",E379,1)+1,(FIND("″",E379,1)-FIND("′",E379,1))-1)</f>
+        <v>28</v>
+      </c>
+      <c r="M379" s="1" t="str">
+        <f t="shared" ref="M379:M387" si="69">MID(F379,1,FIND("°",F379,1)-1)</f>
+        <v>86</v>
+      </c>
+      <c r="N379" s="1" t="str">
+        <f t="shared" ref="N379:N387" si="70">MID(F379,FIND("°",F379,1)+1,(FIND("′",F379,1)-FIND("°",F379,1))-1)</f>
+        <v>06</v>
+      </c>
+      <c r="O379" s="1" t="str">
+        <f t="shared" ref="O379:O387" si="71">MID(F379,FIND("′",F379,1)+1,(FIND("″",F379,1)-FIND("′",F379,1))-1)</f>
+        <v>54</v>
+      </c>
+      <c r="P379" s="2">
+        <f t="shared" ref="P379:P387" si="72">((((L379/60)+K379)/60)+J379)*IF(C379="S",-1, 1)</f>
+        <v>21.157777777777778</v>
+      </c>
+      <c r="Q379" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.114999999999995</v>
+      </c>
+      <c r="R379" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="380" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A380" s="1">
+        <v>379</v>
+      </c>
+      <c r="B380" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C380" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D380" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E380" s="20" t="s">
+        <v>645</v>
+      </c>
+      <c r="F380" s="20" t="s">
+        <v>654</v>
+      </c>
+      <c r="G380" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H380" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I380" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J380" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>21</v>
+      </c>
+      <c r="K380" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>05</v>
+      </c>
+      <c r="L380" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>58</v>
+      </c>
+      <c r="M380" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>85</v>
+      </c>
+      <c r="N380" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>45</v>
+      </c>
+      <c r="O380" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>38</v>
+      </c>
+      <c r="P380" s="2">
+        <f t="shared" si="72"/>
+        <v>21.099444444444444</v>
+      </c>
+      <c r="Q380" s="2">
+        <f t="shared" si="65"/>
+        <v>-85.760555555555555</v>
+      </c>
+      <c r="R380" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="381" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A381" s="1">
+        <v>380</v>
+      </c>
+      <c r="B381" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C381" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D381" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E381" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="F381" s="20" t="s">
+        <v>653</v>
+      </c>
+      <c r="G381" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H381" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I381" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J381" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>21</v>
+      </c>
+      <c r="K381" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>36</v>
+      </c>
+      <c r="L381" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>50</v>
+      </c>
+      <c r="M381" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>86</v>
+      </c>
+      <c r="N381" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>17</v>
+      </c>
+      <c r="O381" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>07</v>
+      </c>
+      <c r="P381" s="2">
+        <f t="shared" si="72"/>
+        <v>21.613888888888887</v>
+      </c>
+      <c r="Q381" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.285277777777779</v>
+      </c>
+      <c r="R381" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="382" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A382" s="1">
+        <v>381</v>
+      </c>
+      <c r="B382" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C382" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D382" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E382" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="F382" s="20" t="s">
+        <v>652</v>
+      </c>
+      <c r="G382" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H382" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I382" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J382" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>21</v>
+      </c>
+      <c r="K382" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>35</v>
+      </c>
+      <c r="L382" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>49</v>
+      </c>
+      <c r="M382" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>86</v>
+      </c>
+      <c r="N382" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>07</v>
+      </c>
+      <c r="O382" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>40</v>
+      </c>
+      <c r="P382" s="2">
+        <f t="shared" si="72"/>
+        <v>21.596944444444446</v>
+      </c>
+      <c r="Q382" s="2">
+        <f t="shared" si="65"/>
+        <v>-86.12777777777778</v>
+      </c>
+      <c r="R382" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="383" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A383" s="1">
+        <v>382</v>
+      </c>
+      <c r="B383" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C383" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D383" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E383" s="20" t="s">
+        <v>648</v>
+      </c>
+      <c r="F383" s="20" t="s">
+        <v>651</v>
+      </c>
+      <c r="G383" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H383" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I383" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J383" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>21</v>
+      </c>
+      <c r="K383" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>34</v>
+      </c>
+      <c r="L383" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>51</v>
+      </c>
+      <c r="M383" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>85</v>
+      </c>
+      <c r="N383" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>59</v>
+      </c>
+      <c r="O383" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>26</v>
+      </c>
+      <c r="P383" s="2">
+        <f t="shared" si="72"/>
+        <v>21.580833333333334</v>
+      </c>
+      <c r="Q383" s="2">
+        <f t="shared" si="65"/>
+        <v>-85.990555555555559</v>
+      </c>
+      <c r="R383" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="384" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A384" s="1">
+        <v>383</v>
+      </c>
+      <c r="B384" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C384" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D384" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E384" s="20" t="s">
+        <v>649</v>
+      </c>
+      <c r="F384" s="20" t="s">
+        <v>650</v>
+      </c>
+      <c r="G384" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="H384" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I384" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="J384" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>21</v>
+      </c>
+      <c r="K384" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>29</v>
+      </c>
+      <c r="L384" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>14</v>
+      </c>
+      <c r="M384" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>85</v>
+      </c>
+      <c r="N384" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>31</v>
+      </c>
+      <c r="O384" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>58</v>
+      </c>
+      <c r="P384" s="2">
+        <f t="shared" si="72"/>
+        <v>21.487222222222222</v>
+      </c>
+      <c r="Q384" s="2">
+        <f t="shared" si="65"/>
+        <v>-85.532777777777781</v>
+      </c>
+      <c r="R384" s="16" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="385" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A385" s="1">
+        <v>384</v>
+      </c>
+      <c r="B385" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C385" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D385" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E385" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F385" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G385" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="H385" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I385" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="J385" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>20</v>
+      </c>
+      <c r="K385" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>51</v>
+      </c>
+      <c r="L385" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>00</v>
+      </c>
+      <c r="M385" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>86</v>
+      </c>
+      <c r="N385" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>55</v>
+      </c>
+      <c r="O385" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>00</v>
+      </c>
+      <c r="P385" s="2">
+        <f t="shared" si="72"/>
+        <v>20.85</v>
+      </c>
+      <c r="Q385" s="2">
+        <f t="shared" ref="Q385:Q387" si="73">((((O385/60)+N385)/60)+M385)*IF(D385="W",-1, 1)</f>
+        <v>-86.916666666666671</v>
+      </c>
+      <c r="R385" s="16" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="386" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A386" s="1">
+        <v>385</v>
+      </c>
+      <c r="B386" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C386" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D386" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E386" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F386" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G386" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="H386" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I386" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="J386" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>20</v>
+      </c>
+      <c r="K386" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>51</v>
+      </c>
+      <c r="L386" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v>00</v>
+      </c>
+      <c r="M386" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>86</v>
+      </c>
+      <c r="N386" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>55</v>
+      </c>
+      <c r="O386" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v>00</v>
+      </c>
+      <c r="P386" s="2">
+        <f t="shared" si="72"/>
+        <v>20.85</v>
+      </c>
+      <c r="Q386" s="2">
+        <f t="shared" si="73"/>
+        <v>-86.916666666666671</v>
+      </c>
+      <c r="R386" s="16" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="387" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A387" s="1">
+        <v>386</v>
+      </c>
+      <c r="B387" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="C387" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D387" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E387" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="F387" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="G387" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="H387" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I387" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="J387" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v>8</v>
+      </c>
+      <c r="K387" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v>45</v>
+      </c>
+      <c r="L387" s="1" t="e">
+        <f t="shared" si="68"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M387" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v>34</v>
+      </c>
+      <c r="N387" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v>57</v>
+      </c>
+      <c r="O387" s="1" t="e">
+        <f t="shared" si="71"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P387" s="2" t="e">
+        <f t="shared" si="72"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q387" s="2" t="e">
+        <f t="shared" si="73"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="R387" s="16" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="388" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B388" s="18"/>
       <c r="E388" s="10"/>
       <c r="F388" s="10"/>
@@ -23771,7 +27568,7 @@
       <c r="P388" s="2"/>
       <c r="Q388" s="2"/>
     </row>
-    <row r="389" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B389" s="18"/>
       <c r="E389" s="10"/>
       <c r="F389" s="10"/>
@@ -23781,7 +27578,7 @@
       <c r="P389" s="2"/>
       <c r="Q389" s="2"/>
     </row>
-    <row r="390" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B390" s="18"/>
       <c r="E390" s="10"/>
       <c r="F390" s="10"/>
@@ -23791,7 +27588,7 @@
       <c r="P390" s="2"/>
       <c r="Q390" s="2"/>
     </row>
-    <row r="391" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B391" s="18"/>
       <c r="E391" s="10"/>
       <c r="F391" s="10"/>
@@ -23801,7 +27598,7 @@
       <c r="P391" s="2"/>
       <c r="Q391" s="2"/>
     </row>
-    <row r="392" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B392" s="18"/>
       <c r="E392" s="10"/>
       <c r="F392" s="10"/>
@@ -23811,7 +27608,7 @@
       <c r="P392" s="2"/>
       <c r="Q392" s="2"/>
     </row>
-    <row r="393" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B393" s="18"/>
       <c r="E393" s="10"/>
       <c r="F393" s="10"/>
@@ -23821,7 +27618,7 @@
       <c r="P393" s="2"/>
       <c r="Q393" s="2"/>
     </row>
-    <row r="394" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B394" s="18"/>
       <c r="E394" s="10"/>
       <c r="F394" s="10"/>
@@ -23831,7 +27628,7 @@
       <c r="P394" s="2"/>
       <c r="Q394" s="2"/>
     </row>
-    <row r="395" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B395" s="18"/>
       <c r="E395" s="10"/>
       <c r="F395" s="10"/>
@@ -23841,7 +27638,7 @@
       <c r="P395" s="2"/>
       <c r="Q395" s="2"/>
     </row>
-    <row r="396" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B396" s="18"/>
       <c r="E396" s="10"/>
       <c r="F396" s="10"/>
@@ -23851,7 +27648,7 @@
       <c r="P396" s="2"/>
       <c r="Q396" s="2"/>
     </row>
-    <row r="397" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B397" s="18"/>
       <c r="E397" s="10"/>
       <c r="F397" s="10"/>
@@ -23861,7 +27658,7 @@
       <c r="P397" s="2"/>
       <c r="Q397" s="2"/>
     </row>
-    <row r="398" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B398" s="18"/>
       <c r="E398" s="10"/>
       <c r="F398" s="10"/>
@@ -23871,7 +27668,7 @@
       <c r="P398" s="2"/>
       <c r="Q398" s="2"/>
     </row>
-    <row r="399" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B399" s="18"/>
       <c r="E399" s="10"/>
       <c r="F399" s="10"/>
@@ -23881,7 +27678,7 @@
       <c r="P399" s="2"/>
       <c r="Q399" s="2"/>
     </row>
-    <row r="400" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B400" s="18"/>
       <c r="E400" s="10"/>
       <c r="F400" s="10"/>
@@ -24214,7 +28011,7 @@
       <c r="Q440" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:I314" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R387" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Deixando os scripts de alex bons
</commit_message>
<xml_diff>
--- a/Ocorrências Literatura.xlsx
+++ b/Ocorrências Literatura.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cofres Obsidian\Mar Aberto\Laboratório\lagostas_carapaca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8400B9A1-B38A-4811-9329-6CAD12FB2954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BBFB1C-2FAC-448A-BBB6-16F75D7B2968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="135" yWindow="7830" windowWidth="16140" windowHeight="7515" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ocorrências Panulirus" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ocorrências Panulirus'!$A$1:$R$454</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ocorrências Panulirus'!$A$1:$R$481</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4095" uniqueCount="877">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4185" uniqueCount="909">
   <si>
     <t>ID</t>
   </si>
@@ -2832,6 +2832,102 @@
   </si>
   <si>
     <t xml:space="preserve">64°47′42″ </t>
+  </si>
+  <si>
+    <t>LOZANO-ÁLVAREZ, E. (2017)</t>
+  </si>
+  <si>
+    <t>20°50′01″</t>
+  </si>
+  <si>
+    <t>86°52′36″</t>
+  </si>
+  <si>
+    <t>ROBERTSON, D. N. (2009)</t>
+  </si>
+  <si>
+    <t>24°43′39″</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24°42′43″ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">24°42′48″ </t>
+  </si>
+  <si>
+    <t>24°55′35″</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24°56′29″ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">24°57′36″ </t>
+  </si>
+  <si>
+    <t>25°01′34″</t>
+  </si>
+  <si>
+    <t>25°02′37″</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25°07′00″ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">80°21′10″ </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80°22′49″ </t>
+  </si>
+  <si>
+    <t>80°24′42″</t>
+  </si>
+  <si>
+    <t>80°33′12″</t>
+  </si>
+  <si>
+    <t>80°33′40″</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80°35′30″ </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80°59′34″</t>
+  </si>
+  <si>
+    <t>80°57′08″</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80°56′20″</t>
+  </si>
+  <si>
+    <t>Recifes "Jardines"</t>
+  </si>
+  <si>
+    <t>robertson2009</t>
+  </si>
+  <si>
+    <t>robertson2010</t>
+  </si>
+  <si>
+    <t>robertson2011</t>
+  </si>
+  <si>
+    <t>robertson2012</t>
+  </si>
+  <si>
+    <t>robertson2013</t>
+  </si>
+  <si>
+    <t>robertson2014</t>
+  </si>
+  <si>
+    <t>robertson2015</t>
+  </si>
+  <si>
+    <t>robertson2016</t>
+  </si>
+  <si>
+    <t>robertson2017</t>
   </si>
 </sst>
 </file>
@@ -2980,7 +3076,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3040,9 +3136,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3306,7 +3399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R454"/>
+  <dimension ref="A1:R481"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -28023,7 +28116,7 @@
       </c>
     </row>
     <row r="387" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A387" s="21">
+      <c r="A387" s="1">
         <v>386</v>
       </c>
       <c r="B387" s="1" t="s">
@@ -28087,7 +28180,7 @@
       </c>
     </row>
     <row r="388" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A388" s="21">
+      <c r="A388" s="1">
         <v>387</v>
       </c>
       <c r="B388" s="1" t="s">
@@ -28151,7 +28244,7 @@
       </c>
     </row>
     <row r="389" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A389" s="21">
+      <c r="A389" s="1">
         <v>388</v>
       </c>
       <c r="B389" s="1" t="s">
@@ -28179,35 +28272,35 @@
         <v>726</v>
       </c>
       <c r="J389" s="1" t="str">
-        <f t="shared" ref="J389:J437" si="85">MID(E389,1,FIND("°",E389,1)-1)</f>
+        <f t="shared" ref="J389:J412" si="85">MID(E389,1,FIND("°",E389,1)-1)</f>
         <v>18</v>
       </c>
       <c r="K389" s="1" t="str">
-        <f t="shared" ref="K389:K437" si="86">MID(E389,FIND("°",E389,1)+1,(FIND("′",E389,1)-FIND("°",E389,1))-1)</f>
+        <f t="shared" ref="K389:K412" si="86">MID(E389,FIND("°",E389,1)+1,(FIND("′",E389,1)-FIND("°",E389,1))-1)</f>
         <v>55</v>
       </c>
       <c r="L389" s="1" t="str">
-        <f t="shared" ref="L389:L437" si="87">MID(E389,FIND("′",E389,1)+1,(FIND("″",E389,1)-FIND("′",E389,1))-1)</f>
+        <f t="shared" ref="L389:L412" si="87">MID(E389,FIND("′",E389,1)+1,(FIND("″",E389,1)-FIND("′",E389,1))-1)</f>
         <v>00</v>
       </c>
       <c r="M389" s="1" t="str">
-        <f t="shared" ref="M389:M437" si="88">MID(F389,1,FIND("°",F389,1)-1)</f>
+        <f t="shared" ref="M389:M412" si="88">MID(F389,1,FIND("°",F389,1)-1)</f>
         <v>75</v>
       </c>
       <c r="N389" s="1" t="str">
-        <f t="shared" ref="N389:N437" si="89">MID(F389,FIND("°",F389,1)+1,(FIND("′",F389,1)-FIND("°",F389,1))-1)</f>
+        <f t="shared" ref="N389:N412" si="89">MID(F389,FIND("°",F389,1)+1,(FIND("′",F389,1)-FIND("°",F389,1))-1)</f>
         <v>20</v>
       </c>
       <c r="O389" s="1" t="str">
-        <f t="shared" ref="O389:O437" si="90">MID(F389,FIND("′",F389,1)+1,(FIND("″",F389,1)-FIND("′",F389,1))-1)</f>
+        <f t="shared" ref="O389:O412" si="90">MID(F389,FIND("′",F389,1)+1,(FIND("″",F389,1)-FIND("′",F389,1))-1)</f>
         <v>00</v>
       </c>
       <c r="P389" s="2">
-        <f t="shared" ref="P389:P437" si="91">((((L389/60)+K389)/60)+J389)*IF(C389="S",-1, 1)</f>
+        <f t="shared" ref="P389:P412" si="91">((((L389/60)+K389)/60)+J389)*IF(C389="S",-1, 1)</f>
         <v>18.916666666666668</v>
       </c>
       <c r="Q389" s="2">
-        <f t="shared" ref="Q389:Q437" si="92">((((O389/60)+N389)/60)+M389)*IF(D389="W",-1, 1)</f>
+        <f t="shared" ref="Q389:Q412" si="92">((((O389/60)+N389)/60)+M389)*IF(D389="W",-1, 1)</f>
         <v>-75.333333333333329</v>
       </c>
       <c r="R389" s="16" t="s">
@@ -28215,7 +28308,7 @@
       </c>
     </row>
     <row r="390" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A390" s="21">
+      <c r="A390" s="1">
         <v>389</v>
       </c>
       <c r="B390" s="1" t="s">
@@ -28279,7 +28372,7 @@
       </c>
     </row>
     <row r="391" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A391" s="21">
+      <c r="A391" s="1">
         <v>390</v>
       </c>
       <c r="B391" s="1" t="s">
@@ -28343,7 +28436,7 @@
       </c>
     </row>
     <row r="392" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A392" s="21">
+      <c r="A392" s="1">
         <v>391</v>
       </c>
       <c r="B392" s="1" t="s">
@@ -28407,7 +28500,7 @@
       </c>
     </row>
     <row r="393" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A393" s="21">
+      <c r="A393" s="1">
         <v>392</v>
       </c>
       <c r="B393" s="1" t="s">
@@ -28471,7 +28564,7 @@
       </c>
     </row>
     <row r="394" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A394" s="21">
+      <c r="A394" s="1">
         <v>393</v>
       </c>
       <c r="B394" s="1" t="s">
@@ -28535,7 +28628,7 @@
       </c>
     </row>
     <row r="395" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A395" s="21">
+      <c r="A395" s="1">
         <v>394</v>
       </c>
       <c r="B395" s="1" t="s">
@@ -28599,7 +28692,7 @@
       </c>
     </row>
     <row r="396" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A396" s="21">
+      <c r="A396" s="1">
         <v>395</v>
       </c>
       <c r="B396" s="1" t="s">
@@ -28663,7 +28756,7 @@
       </c>
     </row>
     <row r="397" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A397" s="21">
+      <c r="A397" s="1">
         <v>396</v>
       </c>
       <c r="B397" s="1" t="s">
@@ -28727,7 +28820,7 @@
       </c>
     </row>
     <row r="398" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A398" s="21">
+      <c r="A398" s="1">
         <v>397</v>
       </c>
       <c r="B398" s="1" t="s">
@@ -28791,7 +28884,7 @@
       </c>
     </row>
     <row r="399" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A399" s="21">
+      <c r="A399" s="1">
         <v>398</v>
       </c>
       <c r="B399" s="1" t="s">
@@ -28855,7 +28948,7 @@
       </c>
     </row>
     <row r="400" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A400" s="21">
+      <c r="A400" s="1">
         <v>399</v>
       </c>
       <c r="B400" s="1" t="s">
@@ -28919,7 +29012,7 @@
       </c>
     </row>
     <row r="401" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A401" s="21">
+      <c r="A401" s="1">
         <v>400</v>
       </c>
       <c r="B401" s="1" t="s">
@@ -28983,7 +29076,7 @@
       </c>
     </row>
     <row r="402" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A402" s="21">
+      <c r="A402" s="1">
         <v>401</v>
       </c>
       <c r="B402" s="1" t="s">
@@ -29047,7 +29140,7 @@
       </c>
     </row>
     <row r="403" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A403" s="21">
+      <c r="A403" s="1">
         <v>402</v>
       </c>
       <c r="B403" s="1" t="s">
@@ -29111,7 +29204,7 @@
       </c>
     </row>
     <row r="404" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A404" s="21">
+      <c r="A404" s="1">
         <v>403</v>
       </c>
       <c r="B404" s="1" t="s">
@@ -29175,7 +29268,7 @@
       </c>
     </row>
     <row r="405" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A405" s="21">
+      <c r="A405" s="1">
         <v>404</v>
       </c>
       <c r="B405" s="1" t="s">
@@ -29239,7 +29332,7 @@
       </c>
     </row>
     <row r="406" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A406" s="21">
+      <c r="A406" s="1">
         <v>405</v>
       </c>
       <c r="B406" s="1" t="s">
@@ -29303,7 +29396,7 @@
       </c>
     </row>
     <row r="407" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A407" s="21">
+      <c r="A407" s="1">
         <v>406</v>
       </c>
       <c r="B407" s="1" t="s">
@@ -29367,7 +29460,7 @@
       </c>
     </row>
     <row r="408" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A408" s="21">
+      <c r="A408" s="1">
         <v>407</v>
       </c>
       <c r="B408" s="1" t="s">
@@ -29431,7 +29524,7 @@
       </c>
     </row>
     <row r="409" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A409" s="21">
+      <c r="A409" s="1">
         <v>408</v>
       </c>
       <c r="B409" s="1" t="s">
@@ -29495,7 +29588,7 @@
       </c>
     </row>
     <row r="410" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A410" s="21">
+      <c r="A410" s="1">
         <v>409</v>
       </c>
       <c r="B410" s="1" t="s">
@@ -29559,7 +29652,7 @@
       </c>
     </row>
     <row r="411" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A411" s="21">
+      <c r="A411" s="1">
         <v>410</v>
       </c>
       <c r="B411" s="1" t="s">
@@ -29623,7 +29716,7 @@
       </c>
     </row>
     <row r="412" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A412" s="21">
+      <c r="A412" s="1">
         <v>411</v>
       </c>
       <c r="B412" s="1" t="s">
@@ -29687,7 +29780,7 @@
       </c>
     </row>
     <row r="413" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A413" s="21">
+      <c r="A413" s="1">
         <v>412</v>
       </c>
       <c r="B413" s="1" t="s">
@@ -29751,7 +29844,7 @@
       </c>
     </row>
     <row r="414" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A414" s="21">
+      <c r="A414" s="1">
         <v>413</v>
       </c>
       <c r="B414" s="1" t="s">
@@ -29815,7 +29908,7 @@
       </c>
     </row>
     <row r="415" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A415" s="21">
+      <c r="A415" s="1">
         <v>414</v>
       </c>
       <c r="B415" s="1" t="s">
@@ -29879,7 +29972,7 @@
       </c>
     </row>
     <row r="416" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A416" s="21">
+      <c r="A416" s="1">
         <v>415</v>
       </c>
       <c r="B416" s="1" t="s">
@@ -29943,7 +30036,7 @@
       </c>
     </row>
     <row r="417" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A417" s="21">
+      <c r="A417" s="1">
         <v>416</v>
       </c>
       <c r="B417" s="1" t="s">
@@ -30007,7 +30100,7 @@
       </c>
     </row>
     <row r="418" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A418" s="21">
+      <c r="A418" s="1">
         <v>417</v>
       </c>
       <c r="B418" s="1" t="s">
@@ -30071,7 +30164,7 @@
       </c>
     </row>
     <row r="419" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A419" s="21">
+      <c r="A419" s="1">
         <v>418</v>
       </c>
       <c r="B419" s="1" t="s">
@@ -30135,7 +30228,7 @@
       </c>
     </row>
     <row r="420" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A420" s="21">
+      <c r="A420" s="1">
         <v>419</v>
       </c>
       <c r="B420" s="1" t="s">
@@ -30199,7 +30292,7 @@
       </c>
     </row>
     <row r="421" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A421" s="21">
+      <c r="A421" s="1">
         <v>420</v>
       </c>
       <c r="B421" s="1" t="s">
@@ -30263,7 +30356,7 @@
       </c>
     </row>
     <row r="422" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A422" s="21">
+      <c r="A422" s="1">
         <v>421</v>
       </c>
       <c r="B422" s="1" t="s">
@@ -30327,7 +30420,7 @@
       </c>
     </row>
     <row r="423" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A423" s="21">
+      <c r="A423" s="1">
         <v>422</v>
       </c>
       <c r="B423" s="1" t="s">
@@ -30391,7 +30484,7 @@
       </c>
     </row>
     <row r="424" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A424" s="21">
+      <c r="A424" s="1">
         <v>423</v>
       </c>
       <c r="B424" s="1" t="s">
@@ -30455,7 +30548,7 @@
       </c>
     </row>
     <row r="425" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A425" s="21">
+      <c r="A425" s="1">
         <v>424</v>
       </c>
       <c r="B425" s="1" t="s">
@@ -30519,7 +30612,7 @@
       </c>
     </row>
     <row r="426" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A426" s="21">
+      <c r="A426" s="1">
         <v>425</v>
       </c>
       <c r="B426" s="1" t="s">
@@ -30583,7 +30676,7 @@
       </c>
     </row>
     <row r="427" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A427" s="21">
+      <c r="A427" s="1">
         <v>426</v>
       </c>
       <c r="B427" s="1" t="s">
@@ -30647,7 +30740,7 @@
       </c>
     </row>
     <row r="428" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A428" s="21">
+      <c r="A428" s="1">
         <v>427</v>
       </c>
       <c r="B428" s="1" t="s">
@@ -30711,7 +30804,7 @@
       </c>
     </row>
     <row r="429" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A429" s="21">
+      <c r="A429" s="1">
         <v>428</v>
       </c>
       <c r="B429" s="1" t="s">
@@ -30775,7 +30868,7 @@
       </c>
     </row>
     <row r="430" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A430" s="21">
+      <c r="A430" s="1">
         <v>429</v>
       </c>
       <c r="B430" s="1" t="s">
@@ -30839,7 +30932,7 @@
       </c>
     </row>
     <row r="431" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A431" s="21">
+      <c r="A431" s="1">
         <v>430</v>
       </c>
       <c r="B431" s="1" t="s">
@@ -30903,7 +30996,7 @@
       </c>
     </row>
     <row r="432" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A432" s="21">
+      <c r="A432" s="1">
         <v>431</v>
       </c>
       <c r="B432" s="1" t="s">
@@ -30967,7 +31060,7 @@
       </c>
     </row>
     <row r="433" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A433" s="21">
+      <c r="A433" s="1">
         <v>432</v>
       </c>
       <c r="B433" s="1" t="s">
@@ -31031,7 +31124,7 @@
       </c>
     </row>
     <row r="434" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A434" s="21">
+      <c r="A434" s="1">
         <v>433</v>
       </c>
       <c r="B434" s="1" t="s">
@@ -31095,7 +31188,7 @@
       </c>
     </row>
     <row r="435" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A435" s="21">
+      <c r="A435" s="1">
         <v>434</v>
       </c>
       <c r="B435" s="1" t="s">
@@ -31159,7 +31252,7 @@
       </c>
     </row>
     <row r="436" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A436" s="21">
+      <c r="A436" s="1">
         <v>435</v>
       </c>
       <c r="B436" s="1" t="s">
@@ -31223,7 +31316,7 @@
       </c>
     </row>
     <row r="437" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A437" s="21">
+      <c r="A437" s="1">
         <v>436</v>
       </c>
       <c r="B437" s="1" t="s">
@@ -31287,7 +31380,7 @@
       </c>
     </row>
     <row r="438" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A438" s="21">
+      <c r="A438" s="1">
         <v>437</v>
       </c>
       <c r="B438" s="1" t="s">
@@ -31351,7 +31444,7 @@
       </c>
     </row>
     <row r="439" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A439" s="21">
+      <c r="A439" s="1">
         <v>438</v>
       </c>
       <c r="B439" s="1" t="s">
@@ -31415,7 +31508,7 @@
       </c>
     </row>
     <row r="440" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A440" s="21">
+      <c r="A440" s="1">
         <v>439</v>
       </c>
       <c r="B440" s="1" t="s">
@@ -31479,7 +31572,7 @@
       </c>
     </row>
     <row r="441" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A441" s="21">
+      <c r="A441" s="1">
         <v>440</v>
       </c>
       <c r="B441" s="1" t="s">
@@ -31543,7 +31636,7 @@
       </c>
     </row>
     <row r="442" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A442" s="21">
+      <c r="A442" s="1">
         <v>441</v>
       </c>
       <c r="B442" s="1" t="s">
@@ -31607,7 +31700,7 @@
       </c>
     </row>
     <row r="443" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A443" s="21">
+      <c r="A443" s="1">
         <v>442</v>
       </c>
       <c r="B443" s="1" t="s">
@@ -31671,7 +31764,7 @@
       </c>
     </row>
     <row r="444" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A444" s="21">
+      <c r="A444" s="1">
         <v>443</v>
       </c>
       <c r="B444" s="1" t="s">
@@ -31735,7 +31828,7 @@
       </c>
     </row>
     <row r="445" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A445" s="21">
+      <c r="A445" s="1">
         <v>444</v>
       </c>
       <c r="B445" s="1" t="s">
@@ -31799,7 +31892,7 @@
       </c>
     </row>
     <row r="446" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A446" s="21">
+      <c r="A446" s="1">
         <v>445</v>
       </c>
       <c r="B446" s="1" t="s">
@@ -31863,7 +31956,7 @@
       </c>
     </row>
     <row r="447" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A447" s="21">
+      <c r="A447" s="1">
         <v>446</v>
       </c>
       <c r="B447" s="1" t="s">
@@ -31927,7 +32020,7 @@
       </c>
     </row>
     <row r="448" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A448" s="21">
+      <c r="A448" s="1">
         <v>447</v>
       </c>
       <c r="B448" s="1" t="s">
@@ -31991,7 +32084,7 @@
       </c>
     </row>
     <row r="449" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A449" s="21">
+      <c r="A449" s="1">
         <v>448</v>
       </c>
       <c r="B449" s="1" t="s">
@@ -32055,7 +32148,7 @@
       </c>
     </row>
     <row r="450" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A450" s="21">
+      <c r="A450" s="1">
         <v>449</v>
       </c>
       <c r="B450" s="1" t="s">
@@ -32119,7 +32212,7 @@
       </c>
     </row>
     <row r="451" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A451" s="21">
+      <c r="A451" s="1">
         <v>450</v>
       </c>
       <c r="B451" s="1" t="s">
@@ -32183,7 +32276,7 @@
       </c>
     </row>
     <row r="452" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A452" s="21">
+      <c r="A452" s="1">
         <v>451</v>
       </c>
       <c r="B452" s="1" t="s">
@@ -32247,7 +32340,7 @@
       </c>
     </row>
     <row r="453" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A453" s="21">
+      <c r="A453" s="1">
         <v>452</v>
       </c>
       <c r="B453" s="1" t="s">
@@ -32311,7 +32404,7 @@
       </c>
     </row>
     <row r="454" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A454" s="21">
+      <c r="A454" s="1">
         <v>453</v>
       </c>
       <c r="B454" s="1" t="s">
@@ -32374,8 +32467,1238 @@
         <v>796</v>
       </c>
     </row>
+    <row r="455" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A455" s="1">
+        <v>454</v>
+      </c>
+      <c r="B455" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C455" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D455" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E455" s="19" t="s">
+        <v>878</v>
+      </c>
+      <c r="F455" s="19" t="s">
+        <v>879</v>
+      </c>
+      <c r="G455" s="19" t="s">
+        <v>877</v>
+      </c>
+      <c r="H455" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I455" s="19" t="s">
+        <v>899</v>
+      </c>
+      <c r="J455" s="1" t="str">
+        <f t="shared" ref="J455:J462" si="115">MID(E455,1,FIND("°",E455,1)-1)</f>
+        <v>20</v>
+      </c>
+      <c r="K455" s="1" t="str">
+        <f t="shared" ref="K455:K462" si="116">MID(E455,FIND("°",E455,1)+1,(FIND("′",E455,1)-FIND("°",E455,1))-1)</f>
+        <v>50</v>
+      </c>
+      <c r="L455" s="1" t="str">
+        <f t="shared" ref="L455:L462" si="117">MID(E455,FIND("′",E455,1)+1,(FIND("″",E455,1)-FIND("′",E455,1))-1)</f>
+        <v>01</v>
+      </c>
+      <c r="M455" s="1" t="str">
+        <f t="shared" ref="M455:M462" si="118">MID(F455,1,FIND("°",F455,1)-1)</f>
+        <v>86</v>
+      </c>
+      <c r="N455" s="1" t="str">
+        <f t="shared" ref="N455:N462" si="119">MID(F455,FIND("°",F455,1)+1,(FIND("′",F455,1)-FIND("°",F455,1))-1)</f>
+        <v>52</v>
+      </c>
+      <c r="O455" s="1" t="str">
+        <f t="shared" ref="O455:O462" si="120">MID(F455,FIND("′",F455,1)+1,(FIND("″",F455,1)-FIND("′",F455,1))-1)</f>
+        <v>36</v>
+      </c>
+      <c r="P455" s="2">
+        <f t="shared" ref="P455:P462" si="121">((((L455/60)+K455)/60)+J455)*IF(C455="S",-1, 1)</f>
+        <v>20.833611111111111</v>
+      </c>
+      <c r="Q455" s="2">
+        <f t="shared" ref="Q455:Q462" si="122">((((O455/60)+N455)/60)+M455)*IF(D455="W",-1, 1)</f>
+        <v>-86.876666666666665</v>
+      </c>
+      <c r="R455" s="16" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="456" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A456" s="1">
+        <v>455</v>
+      </c>
+      <c r="B456" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C456" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D456" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E456" s="2" t="s">
+        <v>881</v>
+      </c>
+      <c r="F456" s="2" t="s">
+        <v>898</v>
+      </c>
+      <c r="G456" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H456" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I456" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J456" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>24</v>
+      </c>
+      <c r="K456" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>43</v>
+      </c>
+      <c r="L456" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>39</v>
+      </c>
+      <c r="M456" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v xml:space="preserve"> 80</v>
+      </c>
+      <c r="N456" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>56</v>
+      </c>
+      <c r="O456" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>20</v>
+      </c>
+      <c r="P456" s="2">
+        <f t="shared" si="121"/>
+        <v>24.727499999999999</v>
+      </c>
+      <c r="Q456" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.938888888888883</v>
+      </c>
+      <c r="R456" s="16" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="457" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A457" s="1">
+        <v>456</v>
+      </c>
+      <c r="B457" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C457" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D457" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E457" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="F457" s="2" t="s">
+        <v>897</v>
+      </c>
+      <c r="G457" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H457" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I457" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J457" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>24</v>
+      </c>
+      <c r="K457" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>42</v>
+      </c>
+      <c r="L457" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>43</v>
+      </c>
+      <c r="M457" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v>80</v>
+      </c>
+      <c r="N457" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>57</v>
+      </c>
+      <c r="O457" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>08</v>
+      </c>
+      <c r="P457" s="2">
+        <f t="shared" si="121"/>
+        <v>24.711944444444445</v>
+      </c>
+      <c r="Q457" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.952222222222218</v>
+      </c>
+      <c r="R457" s="16" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="458" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A458" s="1">
+        <v>457</v>
+      </c>
+      <c r="B458" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C458" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D458" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E458" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="F458" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="G458" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H458" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I458" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J458" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>24</v>
+      </c>
+      <c r="K458" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>42</v>
+      </c>
+      <c r="L458" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>48</v>
+      </c>
+      <c r="M458" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v xml:space="preserve"> 80</v>
+      </c>
+      <c r="N458" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>59</v>
+      </c>
+      <c r="O458" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>34</v>
+      </c>
+      <c r="P458" s="2">
+        <f t="shared" si="121"/>
+        <v>24.713333333333335</v>
+      </c>
+      <c r="Q458" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.992777777777775</v>
+      </c>
+      <c r="R458" s="16" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="459" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A459" s="1">
+        <v>458</v>
+      </c>
+      <c r="B459" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C459" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D459" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E459" s="2" t="s">
+        <v>884</v>
+      </c>
+      <c r="F459" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="G459" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H459" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I459" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J459" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>24</v>
+      </c>
+      <c r="K459" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>55</v>
+      </c>
+      <c r="L459" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>35</v>
+      </c>
+      <c r="M459" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v xml:space="preserve"> 80</v>
+      </c>
+      <c r="N459" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>35</v>
+      </c>
+      <c r="O459" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>30</v>
+      </c>
+      <c r="P459" s="2">
+        <f t="shared" si="121"/>
+        <v>24.926388888888887</v>
+      </c>
+      <c r="Q459" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.591666666666669</v>
+      </c>
+      <c r="R459" s="16" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="460" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A460" s="1">
+        <v>459</v>
+      </c>
+      <c r="B460" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C460" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D460" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E460" s="2" t="s">
+        <v>885</v>
+      </c>
+      <c r="F460" s="2" t="s">
+        <v>894</v>
+      </c>
+      <c r="G460" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H460" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I460" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J460" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>24</v>
+      </c>
+      <c r="K460" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>56</v>
+      </c>
+      <c r="L460" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>29</v>
+      </c>
+      <c r="M460" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v>80</v>
+      </c>
+      <c r="N460" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>33</v>
+      </c>
+      <c r="O460" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>40</v>
+      </c>
+      <c r="P460" s="2">
+        <f t="shared" si="121"/>
+        <v>24.941388888888888</v>
+      </c>
+      <c r="Q460" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.561111111111117</v>
+      </c>
+      <c r="R460" s="16" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="461" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A461" s="1">
+        <v>460</v>
+      </c>
+      <c r="B461" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C461" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D461" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E461" s="2" t="s">
+        <v>886</v>
+      </c>
+      <c r="F461" s="2" t="s">
+        <v>893</v>
+      </c>
+      <c r="G461" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H461" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I461" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J461" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>24</v>
+      </c>
+      <c r="K461" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>57</v>
+      </c>
+      <c r="L461" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>36</v>
+      </c>
+      <c r="M461" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v>80</v>
+      </c>
+      <c r="N461" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>33</v>
+      </c>
+      <c r="O461" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>12</v>
+      </c>
+      <c r="P461" s="2">
+        <f t="shared" si="121"/>
+        <v>24.96</v>
+      </c>
+      <c r="Q461" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.553333333333327</v>
+      </c>
+      <c r="R461" s="16" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="462" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A462" s="1">
+        <v>461</v>
+      </c>
+      <c r="B462" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C462" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D462" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E462" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="F462" s="2" t="s">
+        <v>892</v>
+      </c>
+      <c r="G462" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H462" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I462" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J462" s="1" t="str">
+        <f t="shared" si="115"/>
+        <v>25</v>
+      </c>
+      <c r="K462" s="1" t="str">
+        <f t="shared" si="116"/>
+        <v>01</v>
+      </c>
+      <c r="L462" s="1" t="str">
+        <f t="shared" si="117"/>
+        <v>34</v>
+      </c>
+      <c r="M462" s="1" t="str">
+        <f t="shared" si="118"/>
+        <v>80</v>
+      </c>
+      <c r="N462" s="1" t="str">
+        <f t="shared" si="119"/>
+        <v>24</v>
+      </c>
+      <c r="O462" s="1" t="str">
+        <f t="shared" si="120"/>
+        <v>42</v>
+      </c>
+      <c r="P462" s="2">
+        <f t="shared" si="121"/>
+        <v>25.02611111111111</v>
+      </c>
+      <c r="Q462" s="2">
+        <f t="shared" si="122"/>
+        <v>-80.411666666666662</v>
+      </c>
+      <c r="R462" s="16" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="463" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A463" s="1">
+        <v>462</v>
+      </c>
+      <c r="B463" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C463" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D463" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E463" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="F463" s="2" t="s">
+        <v>891</v>
+      </c>
+      <c r="G463" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H463" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I463" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J463" s="1" t="str">
+        <f t="shared" ref="J463:J481" si="123">MID(E463,1,FIND("°",E463,1)-1)</f>
+        <v>25</v>
+      </c>
+      <c r="K463" s="1" t="str">
+        <f t="shared" ref="K463:K481" si="124">MID(E463,FIND("°",E463,1)+1,(FIND("′",E463,1)-FIND("°",E463,1))-1)</f>
+        <v>02</v>
+      </c>
+      <c r="L463" s="1" t="str">
+        <f t="shared" ref="L463:L481" si="125">MID(E463,FIND("′",E463,1)+1,(FIND("″",E463,1)-FIND("′",E463,1))-1)</f>
+        <v>37</v>
+      </c>
+      <c r="M463" s="1" t="str">
+        <f t="shared" ref="M463:M481" si="126">MID(F463,1,FIND("°",F463,1)-1)</f>
+        <v xml:space="preserve"> 80</v>
+      </c>
+      <c r="N463" s="1" t="str">
+        <f t="shared" ref="N463:N481" si="127">MID(F463,FIND("°",F463,1)+1,(FIND("′",F463,1)-FIND("°",F463,1))-1)</f>
+        <v>22</v>
+      </c>
+      <c r="O463" s="1" t="str">
+        <f t="shared" ref="O463:O481" si="128">MID(F463,FIND("′",F463,1)+1,(FIND("″",F463,1)-FIND("′",F463,1))-1)</f>
+        <v>49</v>
+      </c>
+      <c r="P463" s="2">
+        <f t="shared" ref="P463:P481" si="129">((((L463/60)+K463)/60)+J463)*IF(C463="S",-1, 1)</f>
+        <v>25.043611111111112</v>
+      </c>
+      <c r="Q463" s="2">
+        <f t="shared" ref="Q463:Q481" si="130">((((O463/60)+N463)/60)+M463)*IF(D463="W",-1, 1)</f>
+        <v>-80.380277777777778</v>
+      </c>
+      <c r="R463" s="16" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="464" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A464" s="1">
+        <v>463</v>
+      </c>
+      <c r="B464" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C464" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D464" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E464" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="F464" s="2" t="s">
+        <v>890</v>
+      </c>
+      <c r="G464" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="H464" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I464" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="J464" s="1" t="str">
+        <f t="shared" si="123"/>
+        <v>25</v>
+      </c>
+      <c r="K464" s="1" t="str">
+        <f t="shared" si="124"/>
+        <v>07</v>
+      </c>
+      <c r="L464" s="1" t="str">
+        <f t="shared" si="125"/>
+        <v>00</v>
+      </c>
+      <c r="M464" s="1" t="str">
+        <f t="shared" si="126"/>
+        <v>80</v>
+      </c>
+      <c r="N464" s="1" t="str">
+        <f t="shared" si="127"/>
+        <v>21</v>
+      </c>
+      <c r="O464" s="1" t="str">
+        <f t="shared" si="128"/>
+        <v>10</v>
+      </c>
+      <c r="P464" s="2">
+        <f t="shared" si="129"/>
+        <v>25.116666666666667</v>
+      </c>
+      <c r="Q464" s="2">
+        <f t="shared" si="130"/>
+        <v>-80.352777777777774</v>
+      </c>
+      <c r="R464" s="16" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="465" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G465"/>
+      <c r="J465" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K465" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L465" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M465" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N465" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O465" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P465" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q465" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="466" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G466"/>
+      <c r="J466" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K466" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L466" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M466" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N466" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O466" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P466" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q466" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="467" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G467"/>
+      <c r="J467" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K467" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L467" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M467" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N467" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O467" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P467" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q467" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="468" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G468"/>
+      <c r="J468" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K468" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L468" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M468" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N468" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O468" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P468" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q468" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="469" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G469"/>
+      <c r="J469" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K469" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L469" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M469" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N469" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O469" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P469" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q469" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="470" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G470"/>
+      <c r="J470" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K470" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L470" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M470" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N470" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O470" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P470" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q470" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="471" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G471"/>
+      <c r="J471" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K471" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L471" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M471" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N471" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O471" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P471" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q471" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="472" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G472"/>
+      <c r="J472" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K472" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L472" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M472" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N472" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O472" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P472" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q472" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="473" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G473"/>
+      <c r="J473" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K473" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L473" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M473" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N473" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O473" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P473" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q473" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="474" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G474"/>
+      <c r="J474" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K474" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L474" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M474" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N474" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O474" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P474" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q474" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="475" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G475"/>
+      <c r="J475" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K475" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L475" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M475" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N475" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O475" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P475" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q475" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="476" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G476"/>
+      <c r="J476" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K476" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L476" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M476" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N476" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O476" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P476" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q476" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="477" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="J477" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K477" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L477" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M477" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N477" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O477" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P477" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q477" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="478" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="J478" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K478" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L478" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M478" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N478" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O478" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P478" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q478" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="479" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="J479" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K479" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L479" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M479" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N479" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O479" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P479" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q479" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="480" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="J480" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K480" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L480" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M480" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N480" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O480" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P480" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q480" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="481" spans="10:17" x14ac:dyDescent="0.25">
+      <c r="J481" s="1" t="e">
+        <f t="shared" si="123"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K481" s="1" t="e">
+        <f t="shared" si="124"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L481" s="1" t="e">
+        <f t="shared" si="125"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M481" s="1" t="e">
+        <f t="shared" si="126"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N481" s="1" t="e">
+        <f t="shared" si="127"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="O481" s="1" t="e">
+        <f t="shared" si="128"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P481" s="2" t="e">
+        <f t="shared" si="129"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q481" s="2" t="e">
+        <f t="shared" si="130"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R454" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R481" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>